<commit_message>
BOM: bought power supply
</commit_message>
<xml_diff>
--- a/docs/financials/Buddy_BOM.xlsx
+++ b/docs/financials/Buddy_BOM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ventimaj/Desktop/Buddy_Robot/docs/financials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EC67528-1D7D-7648-B01A-9D76E04AFC14}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95EDD857-862A-CB42-96CD-01D61FA6A83A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29040" windowHeight="15720" xr2:uid="{C64966AC-B3BB-9844-956C-858996BC28CC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="69">
   <si>
     <t>Descriptive Part Name</t>
   </si>
@@ -230,6 +230,24 @@
   </si>
   <si>
     <t>MicroSD to USB-B to USB-A</t>
+  </si>
+  <si>
+    <t>DC Power Supply</t>
+  </si>
+  <si>
+    <t>B0DDPVDWPZ</t>
+  </si>
+  <si>
+    <t>JESVERTY</t>
+  </si>
+  <si>
+    <t>DC Power Supply Variable, 0-32V 0-10A Switching Bench Power Supply with 20W USB &amp; Type-C Quick-Charge, Encoder Corase &amp; Fine Adjustment Knob, Output Switch, 4-Digit LED Display - SPS-3010V</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/dp/B0DDPVDWPZ?smid=A1ESSXTD1TYBDH&amp;ref_=chk_typ_imgToDp&amp;th=1</t>
+  </si>
+  <si>
+    <t>DC Power Supply Variable, 0-32V 0-10A</t>
   </si>
 </sst>
 </file>
@@ -569,7 +587,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -624,9 +642,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -719,6 +734,15 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1268,14 +1292,14 @@
       <c r="Q2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="S2" s="46" t="s">
+      <c r="S2" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="T2" s="46"/>
+      <c r="T2" s="45"/>
       <c r="U2" s="7"/>
     </row>
     <row r="3" spans="2:22" ht="61" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="39" t="s">
         <v>31</v>
       </c>
       <c r="C3" s="16">
@@ -1294,17 +1318,17 @@
       <c r="G3" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="H3" s="35">
+      <c r="H3" s="34">
         <v>46201</v>
       </c>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30" t="s">
+      <c r="I3" s="29"/>
+      <c r="J3" s="29" t="s">
         <v>38</v>
       </c>
       <c r="K3" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="L3" s="30" t="s">
+      <c r="L3" s="29" t="s">
         <v>38</v>
       </c>
       <c r="M3" s="16" t="s">
@@ -1319,7 +1343,7 @@
       <c r="P3" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="Q3" s="32" t="s">
+      <c r="Q3" s="31" t="s">
         <v>41</v>
       </c>
       <c r="S3" s="8"/>
@@ -1328,8 +1352,8 @@
       </c>
       <c r="U3" s="7"/>
     </row>
-    <row r="4" spans="2:22" ht="44" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="40" t="s">
+    <row r="4" spans="2:22" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="39" t="s">
         <v>37</v>
       </c>
       <c r="C4" s="17">
@@ -1348,9 +1372,9 @@
       <c r="G4" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="H4" s="30"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="30" t="s">
+      <c r="H4" s="29"/>
+      <c r="I4" s="29"/>
+      <c r="J4" s="29" t="s">
         <v>18</v>
       </c>
       <c r="K4" s="17" t="s">
@@ -1360,16 +1384,16 @@
         <v>35</v>
       </c>
       <c r="M4" s="17"/>
-      <c r="N4" s="5" t="s">
+      <c r="N4" s="57" t="s">
         <v>36</v>
       </c>
-      <c r="O4" s="25" t="s">
+      <c r="O4" s="24" t="s">
         <v>32</v>
       </c>
-      <c r="P4" s="36" t="s">
+      <c r="P4" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="Q4" s="32" t="s">
+      <c r="Q4" s="31" t="s">
         <v>33</v>
       </c>
       <c r="S4" s="7"/>
@@ -1377,7 +1401,7 @@
       <c r="U4" s="7"/>
     </row>
     <row r="5" spans="2:22" ht="75" x14ac:dyDescent="0.2">
-      <c r="B5" s="41" t="s">
+      <c r="B5" s="40" t="s">
         <v>59</v>
       </c>
       <c r="C5" s="16">
@@ -1396,10 +1420,10 @@
       <c r="G5" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="H5" s="43">
+      <c r="H5" s="42">
         <v>46202</v>
       </c>
-      <c r="I5" s="43">
+      <c r="I5" s="42">
         <v>46205</v>
       </c>
       <c r="J5" s="17"/>
@@ -1407,23 +1431,23 @@
       <c r="L5" s="17"/>
       <c r="M5" s="17"/>
       <c r="N5" s="5"/>
-      <c r="O5" s="25" t="s">
+      <c r="O5" s="24" t="s">
         <v>58</v>
       </c>
       <c r="P5" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="Q5" s="33" t="s">
+      <c r="Q5" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="S5" s="47" t="s">
+      <c r="S5" s="46" t="s">
         <v>21</v>
       </c>
-      <c r="T5" s="47"/>
+      <c r="T5" s="46"/>
       <c r="U5" s="7"/>
     </row>
     <row r="6" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B6" s="40" t="s">
+      <c r="B6" s="39" t="s">
         <v>61</v>
       </c>
       <c r="C6" s="17">
@@ -1440,7 +1464,7 @@
       <c r="G6" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="H6" s="17"/>
+      <c r="H6" s="42"/>
       <c r="I6" s="17"/>
       <c r="J6" s="17"/>
       <c r="K6" s="17"/>
@@ -1448,16 +1472,16 @@
       <c r="M6" s="17"/>
       <c r="N6" s="5"/>
       <c r="O6" s="23"/>
-      <c r="P6" s="37"/>
-      <c r="Q6" s="33"/>
-      <c r="S6" s="44" t="s">
+      <c r="P6" s="36"/>
+      <c r="Q6" s="32"/>
+      <c r="S6" s="43" t="s">
         <v>60</v>
       </c>
-      <c r="T6" s="44"/>
+      <c r="T6" s="43"/>
       <c r="U6" s="7"/>
     </row>
     <row r="7" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B7" s="40" t="s">
+      <c r="B7" s="39" t="s">
         <v>62</v>
       </c>
       <c r="C7" s="16">
@@ -1474,7 +1498,7 @@
       <c r="G7" s="16" t="s">
         <v>60</v>
       </c>
-      <c r="H7" s="17"/>
+      <c r="H7" s="42"/>
       <c r="I7" s="17"/>
       <c r="J7" s="17"/>
       <c r="K7" s="17"/>
@@ -1482,50 +1506,67 @@
       <c r="M7" s="17"/>
       <c r="N7" s="5"/>
       <c r="O7" s="23"/>
-      <c r="P7" s="37"/>
-      <c r="Q7" s="33"/>
-      <c r="S7" s="48" t="s">
+      <c r="P7" s="36"/>
+      <c r="Q7" s="32"/>
+      <c r="S7" s="47" t="s">
         <v>17</v>
       </c>
-      <c r="T7" s="48"/>
+      <c r="T7" s="47"/>
       <c r="U7" s="7"/>
     </row>
-    <row r="8" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B8" s="40" t="s">
-        <v>42</v>
-      </c>
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="19" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+    <row r="8" spans="2:22" ht="60" x14ac:dyDescent="0.2">
+      <c r="B8" s="55" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="17">
+        <v>1</v>
+      </c>
+      <c r="D8" s="17">
+        <v>1</v>
+      </c>
+      <c r="E8" s="18">
+        <v>48.48</v>
+      </c>
+      <c r="F8" s="19">
+        <f t="shared" si="0"/>
+        <v>48.48</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="H8" s="31"/>
-      <c r="I8" s="31"/>
-      <c r="J8" s="31"/>
-      <c r="K8" s="17"/>
-      <c r="L8" s="17"/>
+        <v>23</v>
+      </c>
+      <c r="H8" s="42">
+        <v>46206</v>
+      </c>
+      <c r="I8" s="30"/>
+      <c r="J8" s="30" t="s">
+        <v>18</v>
+      </c>
+      <c r="K8" s="17" t="s">
+        <v>64</v>
+      </c>
+      <c r="L8" s="17" t="s">
+        <v>65</v>
+      </c>
       <c r="M8" s="17"/>
-      <c r="N8" s="5"/>
-      <c r="O8" s="24"/>
-      <c r="P8" s="38" t="s">
+      <c r="N8" s="57" t="s">
+        <v>68</v>
+      </c>
+      <c r="O8" s="56" t="s">
+        <v>67</v>
+      </c>
+      <c r="P8" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="Q8" s="33"/>
-      <c r="S8" s="49" t="s">
+      <c r="Q8" s="31" t="s">
+        <v>66</v>
+      </c>
+      <c r="S8" s="48" t="s">
         <v>19</v>
       </c>
-      <c r="T8" s="49"/>
+      <c r="T8" s="48"/>
       <c r="U8" s="7"/>
     </row>
     <row r="9" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B9" s="40" t="s">
-        <v>43</v>
-      </c>
       <c r="C9" s="16"/>
       <c r="D9" s="17"/>
       <c r="E9" s="18"/>
@@ -1536,7 +1577,7 @@
       <c r="G9" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H9" s="17"/>
+      <c r="H9" s="42"/>
       <c r="I9" s="17"/>
       <c r="J9" s="17"/>
       <c r="K9" s="17"/>
@@ -1544,18 +1585,15 @@
       <c r="M9" s="17"/>
       <c r="N9" s="5"/>
       <c r="O9" s="23"/>
-      <c r="P9" s="37"/>
-      <c r="Q9" s="33"/>
-      <c r="S9" s="50" t="s">
+      <c r="P9" s="36"/>
+      <c r="Q9" s="32"/>
+      <c r="S9" s="49" t="s">
         <v>23</v>
       </c>
-      <c r="T9" s="50"/>
+      <c r="T9" s="49"/>
       <c r="U9" s="7"/>
     </row>
     <row r="10" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B10" s="40" t="s">
-        <v>44</v>
-      </c>
       <c r="C10" s="17"/>
       <c r="D10" s="17"/>
       <c r="E10" s="18"/>
@@ -1566,7 +1604,7 @@
       <c r="G10" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H10" s="17"/>
+      <c r="H10" s="42"/>
       <c r="I10" s="17"/>
       <c r="J10" s="17"/>
       <c r="K10" s="17"/>
@@ -1574,18 +1612,15 @@
       <c r="M10" s="17"/>
       <c r="N10" s="5"/>
       <c r="O10" s="23"/>
-      <c r="P10" s="37"/>
-      <c r="Q10" s="33"/>
-      <c r="S10" s="51" t="s">
+      <c r="P10" s="36"/>
+      <c r="Q10" s="32"/>
+      <c r="S10" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="T10" s="51"/>
+      <c r="T10" s="50"/>
       <c r="U10" s="7"/>
     </row>
     <row r="11" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B11" s="40" t="s">
-        <v>45</v>
-      </c>
       <c r="C11" s="16"/>
       <c r="D11" s="17"/>
       <c r="E11" s="18"/>
@@ -1596,7 +1631,7 @@
       <c r="G11" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H11" s="17"/>
+      <c r="H11" s="42"/>
       <c r="I11" s="17"/>
       <c r="J11" s="17"/>
       <c r="K11" s="17"/>
@@ -1604,18 +1639,15 @@
       <c r="M11" s="17"/>
       <c r="N11" s="5"/>
       <c r="O11" s="23"/>
-      <c r="P11" s="37"/>
-      <c r="Q11" s="33"/>
-      <c r="S11" s="52" t="s">
+      <c r="P11" s="36"/>
+      <c r="Q11" s="32"/>
+      <c r="S11" s="51" t="s">
         <v>25</v>
       </c>
-      <c r="T11" s="52"/>
+      <c r="T11" s="51"/>
       <c r="U11" s="7"/>
     </row>
     <row r="12" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B12" s="40" t="s">
-        <v>46</v>
-      </c>
       <c r="C12" s="17"/>
       <c r="D12" s="17"/>
       <c r="E12" s="18"/>
@@ -1626,7 +1658,7 @@
       <c r="G12" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H12" s="17"/>
+      <c r="H12" s="42"/>
       <c r="I12" s="17"/>
       <c r="J12" s="17"/>
       <c r="K12" s="17"/>
@@ -1634,18 +1666,15 @@
       <c r="M12" s="17"/>
       <c r="N12" s="5"/>
       <c r="O12" s="23"/>
-      <c r="P12" s="37"/>
-      <c r="Q12" s="33"/>
-      <c r="S12" s="53" t="s">
+      <c r="P12" s="36"/>
+      <c r="Q12" s="32"/>
+      <c r="S12" s="52" t="s">
         <v>26</v>
       </c>
-      <c r="T12" s="53"/>
+      <c r="T12" s="52"/>
       <c r="U12" s="7"/>
     </row>
     <row r="13" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B13" s="40" t="s">
-        <v>47</v>
-      </c>
       <c r="C13" s="17"/>
       <c r="D13" s="17"/>
       <c r="E13" s="18"/>
@@ -1656,26 +1685,23 @@
       <c r="G13" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H13" s="30"/>
-      <c r="I13" s="30"/>
-      <c r="J13" s="30"/>
+      <c r="H13" s="42"/>
+      <c r="I13" s="29"/>
+      <c r="J13" s="29"/>
       <c r="K13" s="17"/>
       <c r="L13" s="17"/>
       <c r="M13" s="17"/>
       <c r="N13" s="5"/>
       <c r="O13" s="20"/>
-      <c r="P13" s="36"/>
-      <c r="Q13" s="33"/>
-      <c r="S13" s="54" t="s">
+      <c r="P13" s="35"/>
+      <c r="Q13" s="32"/>
+      <c r="S13" s="53" t="s">
         <v>27</v>
       </c>
-      <c r="T13" s="54"/>
+      <c r="T13" s="53"/>
       <c r="U13" s="7"/>
     </row>
     <row r="14" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B14" s="40" t="s">
-        <v>48</v>
-      </c>
       <c r="C14" s="16"/>
       <c r="D14" s="17"/>
       <c r="E14" s="18"/>
@@ -1686,7 +1712,7 @@
       <c r="G14" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H14" s="17"/>
+      <c r="H14" s="42"/>
       <c r="I14" s="17"/>
       <c r="J14" s="17"/>
       <c r="K14" s="17"/>
@@ -1694,18 +1720,15 @@
       <c r="M14" s="17"/>
       <c r="N14" s="5"/>
       <c r="O14" s="23"/>
-      <c r="P14" s="37"/>
-      <c r="Q14" s="33"/>
-      <c r="S14" s="55" t="s">
+      <c r="P14" s="36"/>
+      <c r="Q14" s="32"/>
+      <c r="S14" s="54" t="s">
         <v>16</v>
       </c>
-      <c r="T14" s="55"/>
+      <c r="T14" s="54"/>
       <c r="U14" s="7"/>
     </row>
     <row r="15" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B15" s="40" t="s">
-        <v>49</v>
-      </c>
       <c r="C15" s="17"/>
       <c r="D15" s="17"/>
       <c r="E15" s="18"/>
@@ -1716,26 +1739,23 @@
       <c r="G15" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H15" s="17"/>
+      <c r="H15" s="42"/>
       <c r="I15" s="17"/>
       <c r="J15" s="17"/>
       <c r="K15" s="17"/>
       <c r="L15" s="17"/>
       <c r="M15" s="17"/>
       <c r="N15" s="5"/>
-      <c r="O15" s="25"/>
+      <c r="O15" s="24"/>
       <c r="P15" s="22"/>
-      <c r="Q15" s="33"/>
-      <c r="S15" s="45" t="s">
-        <v>14</v>
-      </c>
-      <c r="T15" s="45"/>
+      <c r="Q15" s="32"/>
+      <c r="S15" s="44" t="s">
+        <v>14</v>
+      </c>
+      <c r="T15" s="44"/>
       <c r="U15" s="7"/>
     </row>
     <row r="16" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B16" s="40" t="s">
-        <v>50</v>
-      </c>
       <c r="C16" s="17"/>
       <c r="D16" s="17"/>
       <c r="E16" s="18"/>
@@ -1746,23 +1766,20 @@
       <c r="G16" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H16" s="30"/>
-      <c r="I16" s="30"/>
-      <c r="J16" s="30"/>
+      <c r="H16" s="42"/>
+      <c r="I16" s="29"/>
+      <c r="J16" s="29"/>
       <c r="K16" s="17"/>
       <c r="L16" s="17"/>
       <c r="M16" s="17"/>
       <c r="N16" s="5"/>
       <c r="O16" s="20"/>
-      <c r="P16" s="36"/>
-      <c r="Q16" s="33"/>
+      <c r="P16" s="35"/>
+      <c r="Q16" s="32"/>
       <c r="U16" s="7"/>
       <c r="V16" s="7"/>
     </row>
     <row r="17" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B17" s="40" t="s">
-        <v>51</v>
-      </c>
       <c r="C17" s="16"/>
       <c r="D17" s="17"/>
       <c r="E17" s="18"/>
@@ -1773,23 +1790,20 @@
       <c r="G17" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H17" s="17"/>
+      <c r="H17" s="42"/>
       <c r="I17" s="17"/>
       <c r="J17" s="17"/>
       <c r="K17" s="17"/>
       <c r="L17" s="17"/>
       <c r="M17" s="17"/>
       <c r="N17" s="5"/>
-      <c r="O17" s="25"/>
+      <c r="O17" s="24"/>
       <c r="P17" s="22"/>
-      <c r="Q17" s="33"/>
+      <c r="Q17" s="32"/>
       <c r="S17" s="7"/>
       <c r="V17" s="7"/>
     </row>
     <row r="18" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B18" s="40" t="s">
-        <v>52</v>
-      </c>
       <c r="C18" s="17"/>
       <c r="D18" s="17"/>
       <c r="E18" s="18"/>
@@ -1800,7 +1814,7 @@
       <c r="G18" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H18" s="17"/>
+      <c r="H18" s="42"/>
       <c r="I18" s="17"/>
       <c r="J18" s="17"/>
       <c r="K18" s="17"/>
@@ -1808,13 +1822,15 @@
       <c r="M18" s="17"/>
       <c r="N18" s="5"/>
       <c r="O18" s="23"/>
-      <c r="P18" s="37"/>
-      <c r="Q18" s="33"/>
+      <c r="P18" s="36"/>
+      <c r="Q18" s="32"/>
       <c r="S18" s="7"/>
       <c r="V18" s="7"/>
     </row>
     <row r="19" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B19" s="40"/>
+      <c r="B19" s="39" t="s">
+        <v>42</v>
+      </c>
       <c r="C19" s="16"/>
       <c r="D19" s="17"/>
       <c r="E19" s="18"/>
@@ -1825,7 +1841,7 @@
       <c r="G19" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H19" s="17"/>
+      <c r="H19" s="42"/>
       <c r="I19" s="17"/>
       <c r="J19" s="17"/>
       <c r="K19" s="17"/>
@@ -1833,13 +1849,15 @@
       <c r="M19" s="17"/>
       <c r="N19" s="5"/>
       <c r="O19" s="23"/>
-      <c r="P19" s="37"/>
-      <c r="Q19" s="33"/>
+      <c r="P19" s="36"/>
+      <c r="Q19" s="32"/>
       <c r="S19" s="7"/>
       <c r="V19" s="7"/>
     </row>
     <row r="20" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B20" s="40"/>
+      <c r="B20" s="39" t="s">
+        <v>43</v>
+      </c>
       <c r="C20" s="16"/>
       <c r="D20" s="17"/>
       <c r="E20" s="18"/>
@@ -1850,21 +1868,23 @@
       <c r="G20" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H20" s="30"/>
-      <c r="I20" s="30"/>
-      <c r="J20" s="30"/>
+      <c r="H20" s="42"/>
+      <c r="I20" s="29"/>
+      <c r="J20" s="29"/>
       <c r="K20" s="17"/>
       <c r="L20" s="17"/>
       <c r="M20" s="17"/>
       <c r="N20" s="5"/>
       <c r="O20" s="20"/>
-      <c r="P20" s="36"/>
-      <c r="Q20" s="33"/>
+      <c r="P20" s="35"/>
+      <c r="Q20" s="32"/>
       <c r="S20" s="7"/>
       <c r="V20" s="7"/>
     </row>
     <row r="21" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B21" s="40"/>
+      <c r="B21" s="39" t="s">
+        <v>44</v>
+      </c>
       <c r="C21" s="17"/>
       <c r="D21" s="17"/>
       <c r="E21" s="18"/>
@@ -1875,19 +1895,21 @@
       <c r="G21" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H21" s="30"/>
-      <c r="I21" s="30"/>
-      <c r="J21" s="30"/>
+      <c r="H21" s="29"/>
+      <c r="I21" s="29"/>
+      <c r="J21" s="29"/>
       <c r="K21" s="17"/>
       <c r="L21" s="17"/>
       <c r="M21" s="17"/>
       <c r="N21" s="5"/>
       <c r="O21" s="20"/>
-      <c r="P21" s="36"/>
-      <c r="Q21" s="33"/>
+      <c r="P21" s="35"/>
+      <c r="Q21" s="32"/>
     </row>
     <row r="22" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B22" s="40"/>
+      <c r="B22" s="39" t="s">
+        <v>45</v>
+      </c>
       <c r="C22" s="16"/>
       <c r="D22" s="17"/>
       <c r="E22" s="18"/>
@@ -1906,11 +1928,13 @@
       <c r="M22" s="17"/>
       <c r="N22" s="5"/>
       <c r="O22" s="23"/>
-      <c r="P22" s="37"/>
-      <c r="Q22" s="33"/>
+      <c r="P22" s="36"/>
+      <c r="Q22" s="32"/>
     </row>
     <row r="23" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="40"/>
+      <c r="B23" s="39" t="s">
+        <v>46</v>
+      </c>
       <c r="C23" s="17"/>
       <c r="D23" s="17"/>
       <c r="E23" s="18"/>
@@ -1929,11 +1953,13 @@
       <c r="M23" s="17"/>
       <c r="N23" s="5"/>
       <c r="O23" s="20"/>
-      <c r="P23" s="36"/>
-      <c r="Q23" s="33"/>
+      <c r="P23" s="35"/>
+      <c r="Q23" s="32"/>
     </row>
     <row r="24" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B24" s="40"/>
+      <c r="B24" s="39" t="s">
+        <v>47</v>
+      </c>
       <c r="C24" s="16"/>
       <c r="D24" s="17"/>
       <c r="E24" s="18"/>
@@ -1952,8 +1978,8 @@
       <c r="M24" s="17"/>
       <c r="N24" s="5"/>
       <c r="O24" s="20"/>
-      <c r="P24" s="36"/>
-      <c r="Q24" s="33"/>
+      <c r="P24" s="35"/>
+      <c r="Q24" s="32"/>
       <c r="S24" s="10" t="s">
         <v>28</v>
       </c>
@@ -1962,7 +1988,9 @@
       </c>
     </row>
     <row r="25" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="40"/>
+      <c r="B25" s="39" t="s">
+        <v>48</v>
+      </c>
       <c r="C25" s="17"/>
       <c r="D25" s="17"/>
       <c r="E25" s="18"/>
@@ -1973,26 +2001,28 @@
       <c r="G25" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H25" s="30"/>
-      <c r="I25" s="30"/>
-      <c r="J25" s="30"/>
+      <c r="H25" s="29"/>
+      <c r="I25" s="29"/>
+      <c r="J25" s="29"/>
       <c r="K25" s="17"/>
       <c r="L25" s="17"/>
       <c r="M25" s="17"/>
       <c r="N25" s="5"/>
       <c r="O25" s="20"/>
-      <c r="P25" s="36"/>
-      <c r="Q25" s="33"/>
+      <c r="P25" s="35"/>
+      <c r="Q25" s="32"/>
       <c r="S25" s="12" t="s">
         <v>29</v>
       </c>
       <c r="T25" s="13">
         <f>SUM(F3:F37)</f>
-        <v>293.29000000000002</v>
+        <v>341.77000000000004</v>
       </c>
     </row>
     <row r="26" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="40"/>
+      <c r="B26" s="39" t="s">
+        <v>49</v>
+      </c>
       <c r="C26" s="16"/>
       <c r="D26" s="17"/>
       <c r="E26" s="18"/>
@@ -2011,18 +2041,20 @@
       <c r="M26" s="17"/>
       <c r="N26" s="5"/>
       <c r="O26" s="20"/>
-      <c r="P26" s="36"/>
-      <c r="Q26" s="33"/>
+      <c r="P26" s="35"/>
+      <c r="Q26" s="32"/>
       <c r="S26" s="14" t="s">
         <v>30</v>
       </c>
       <c r="T26" s="15">
         <f>T24-T25</f>
-        <v>1706.71</v>
+        <v>1658.23</v>
       </c>
     </row>
     <row r="27" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B27" s="40"/>
+      <c r="B27" s="39" t="s">
+        <v>50</v>
+      </c>
       <c r="C27" s="17"/>
       <c r="D27" s="17"/>
       <c r="E27" s="18"/>
@@ -2041,11 +2073,13 @@
       <c r="M27" s="17"/>
       <c r="N27" s="5"/>
       <c r="O27" s="20"/>
-      <c r="P27" s="36"/>
-      <c r="Q27" s="33"/>
+      <c r="P27" s="35"/>
+      <c r="Q27" s="32"/>
     </row>
     <row r="28" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B28" s="40"/>
+      <c r="B28" s="39" t="s">
+        <v>51</v>
+      </c>
       <c r="C28" s="16"/>
       <c r="D28" s="17"/>
       <c r="E28" s="18"/>
@@ -2064,11 +2098,13 @@
       <c r="M28" s="17"/>
       <c r="N28" s="5"/>
       <c r="O28" s="23"/>
-      <c r="P28" s="37"/>
-      <c r="Q28" s="33"/>
+      <c r="P28" s="36"/>
+      <c r="Q28" s="32"/>
     </row>
     <row r="29" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B29" s="40"/>
+      <c r="B29" s="39" t="s">
+        <v>52</v>
+      </c>
       <c r="C29" s="17"/>
       <c r="D29" s="17"/>
       <c r="E29" s="18"/>
@@ -2087,11 +2123,11 @@
       <c r="M29" s="17"/>
       <c r="N29" s="5"/>
       <c r="O29" s="23"/>
-      <c r="P29" s="37"/>
-      <c r="Q29" s="33"/>
+      <c r="P29" s="36"/>
+      <c r="Q29" s="32"/>
     </row>
     <row r="30" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B30" s="40"/>
+      <c r="B30" s="39"/>
       <c r="C30" s="16"/>
       <c r="D30" s="17"/>
       <c r="E30" s="18"/>
@@ -2110,11 +2146,11 @@
       <c r="M30" s="17"/>
       <c r="N30" s="5"/>
       <c r="O30" s="23"/>
-      <c r="P30" s="37"/>
-      <c r="Q30" s="33"/>
+      <c r="P30" s="36"/>
+      <c r="Q30" s="32"/>
     </row>
     <row r="31" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B31" s="40"/>
+      <c r="B31" s="39"/>
       <c r="C31" s="17"/>
       <c r="D31" s="17"/>
       <c r="E31" s="18"/>
@@ -2133,11 +2169,11 @@
       <c r="M31" s="17"/>
       <c r="N31" s="5"/>
       <c r="O31" s="23"/>
-      <c r="P31" s="37"/>
-      <c r="Q31" s="33"/>
+      <c r="P31" s="36"/>
+      <c r="Q31" s="32"/>
     </row>
     <row r="32" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B32" s="40"/>
+      <c r="B32" s="39"/>
       <c r="C32" s="17"/>
       <c r="D32" s="17"/>
       <c r="E32" s="18"/>
@@ -2156,11 +2192,11 @@
       <c r="M32" s="17"/>
       <c r="N32" s="5"/>
       <c r="O32" s="23"/>
-      <c r="P32" s="37"/>
-      <c r="Q32" s="33"/>
+      <c r="P32" s="36"/>
+      <c r="Q32" s="32"/>
     </row>
     <row r="33" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B33" s="40"/>
+      <c r="B33" s="39"/>
       <c r="C33" s="16"/>
       <c r="D33" s="17"/>
       <c r="E33" s="18"/>
@@ -2179,11 +2215,11 @@
       <c r="M33" s="17"/>
       <c r="N33" s="5"/>
       <c r="O33" s="23"/>
-      <c r="P33" s="37"/>
-      <c r="Q33" s="33"/>
+      <c r="P33" s="36"/>
+      <c r="Q33" s="32"/>
     </row>
     <row r="34" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B34" s="40"/>
+      <c r="B34" s="39"/>
       <c r="C34" s="17"/>
       <c r="D34" s="17"/>
       <c r="E34" s="18"/>
@@ -2202,11 +2238,11 @@
       <c r="M34" s="17"/>
       <c r="N34" s="5"/>
       <c r="O34" s="23"/>
-      <c r="P34" s="37"/>
-      <c r="Q34" s="33"/>
+      <c r="P34" s="36"/>
+      <c r="Q34" s="32"/>
     </row>
     <row r="35" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B35" s="40"/>
+      <c r="B35" s="39"/>
       <c r="C35" s="17"/>
       <c r="D35" s="17"/>
       <c r="E35" s="18"/>
@@ -2225,11 +2261,11 @@
       <c r="M35" s="17"/>
       <c r="N35" s="5"/>
       <c r="O35" s="23"/>
-      <c r="P35" s="37"/>
-      <c r="Q35" s="33"/>
+      <c r="P35" s="36"/>
+      <c r="Q35" s="32"/>
     </row>
     <row r="36" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B36" s="40"/>
+      <c r="B36" s="39"/>
       <c r="C36" s="17"/>
       <c r="D36" s="17"/>
       <c r="E36" s="18"/>
@@ -2248,31 +2284,31 @@
       <c r="M36" s="17"/>
       <c r="N36" s="5"/>
       <c r="O36" s="23"/>
-      <c r="P36" s="37"/>
-      <c r="Q36" s="33"/>
+      <c r="P36" s="36"/>
+      <c r="Q36" s="32"/>
     </row>
     <row r="37" spans="2:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="42"/>
-      <c r="C37" s="26"/>
-      <c r="D37" s="26"/>
-      <c r="E37" s="27"/>
-      <c r="F37" s="28" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="G37" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="H37" s="26"/>
-      <c r="I37" s="26"/>
-      <c r="J37" s="26"/>
-      <c r="K37" s="26"/>
-      <c r="L37" s="26"/>
-      <c r="M37" s="26"/>
+      <c r="B37" s="41"/>
+      <c r="C37" s="25"/>
+      <c r="D37" s="25"/>
+      <c r="E37" s="26"/>
+      <c r="F37" s="27" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="G37" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="H37" s="25"/>
+      <c r="I37" s="25"/>
+      <c r="J37" s="25"/>
+      <c r="K37" s="25"/>
+      <c r="L37" s="25"/>
+      <c r="M37" s="25"/>
       <c r="N37" s="6"/>
-      <c r="O37" s="29"/>
-      <c r="P37" s="39"/>
-      <c r="Q37" s="34"/>
+      <c r="O37" s="28"/>
+      <c r="P37" s="38"/>
+      <c r="Q37" s="33"/>
     </row>
   </sheetData>
   <mergeCells count="12">
@@ -2361,7 +2397,9 @@
     <hyperlink ref="P3" r:id="rId3" xr:uid="{72961FDD-8858-432E-8E2C-06893D7B206D}"/>
     <hyperlink ref="P5" r:id="rId4" xr:uid="{8F840528-6D9F-4456-8BB5-74A65BFEE351}"/>
     <hyperlink ref="O5" r:id="rId5" display="https://vilros.com/products/vilros-soldering-iron-kit-electronics-14-in-1-60w-adjustable-temperature-soldering-iron-with-on-off-switch-5pcs-soldering-iron-tips-desoldering-pump-tweezers-stand-solder-pu-carry-bag?variant=31184817684574&amp;country=US&amp;currency=USD&amp;utm_medium=product_sync&amp;utm_source=google&amp;utm_content=sag_organic&amp;utm_campaign=sag_organic&amp;tw_source=google&amp;tw_adid=&amp;tw_campaign=18070425970&amp;gad_source=1&amp;gad_campaignid=17177576781&amp;gbraid=0AAAAAD1QJAhpwOz4TG9imhRizOjsiF33r&amp;gclid=Cj0KCQjwr4jSBhCSARIsAOX1E-IcDf7VArvc12fU96XQu_eogR6Cku3p0W322S9UE6enAxh-gCdhcRkaApEYEALw_wcB" xr:uid="{F8EE24A7-3DF2-4835-8818-4CF5FD2EFD11}"/>
+    <hyperlink ref="O8" r:id="rId6" xr:uid="{ED02DEDC-B0EC-0749-B7B9-A7D73B4129EF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
BOM: bought adapters, HDMI cables, thumb drive
</commit_message>
<xml_diff>
--- a/docs/financials/Buddy_BOM.xlsx
+++ b/docs/financials/Buddy_BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ventimaj/Desktop/Buddy_Robot/docs/financials/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\venti\Desktop\Buddy_Robot\docs\financials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95EDD857-862A-CB42-96CD-01D61FA6A83A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6010315A-D91F-48F0-9EB4-4B1A3CAF49B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29040" windowHeight="15720" xr2:uid="{C64966AC-B3BB-9844-956C-858996BC28CC}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{C64966AC-B3BB-9844-956C-858996BC28CC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="89">
   <si>
     <t>Descriptive Part Name</t>
   </si>
@@ -248,6 +248,66 @@
   </si>
   <si>
     <t>DC Power Supply Variable, 0-32V 0-10A</t>
+  </si>
+  <si>
+    <t>HDMI Cables, 6ft</t>
+  </si>
+  <si>
+    <t>Amazon Basics HDMI Cable, 3-Pack, 6 ft, High-Speed 4K@60Hz HDMI 2.0 Cord, 18Gbps, 2160p, 48 bit, Compatible with TV/PS5/Xbox/Roku/Blu-ray, Ethernet Ready, Black</t>
+  </si>
+  <si>
+    <t>3-Pack, 6 ft, High-Speed 4K@60Hz HDMI 2.0 Cord, 18Gbps, 2160p, 48 bit</t>
+  </si>
+  <si>
+    <t>https://www.amazon.com/dp/B01H7M6YKI?ref=ppx_yo2ov_dt_b_fed_asin_title&amp;th=1</t>
+  </si>
+  <si>
+    <t>USB &amp; USBC Flashdrive, 128 GB</t>
+  </si>
+  <si>
+    <t>B01H7M6YKI</t>
+  </si>
+  <si>
+    <t>B088LMS5VV</t>
+  </si>
+  <si>
+    <t>Flash Drive 128GB 2 in 1 OTG USB 3.0/Type C</t>
+  </si>
+  <si>
+    <t>Amazon.com: KOOTION USB C Flash Drive 128GB 2 in 1 OTG USB 3.0/Type C Thumb Drive Dual Drive USB C Memory Stick for Smartphone/Laptop/Tablet/PC - 128G, Blue : Electronics</t>
+  </si>
+  <si>
+    <t>KOOTION USB C Flash Drive 128GB 2 in 1 OTG USB 3.0/Type C Thumb Drive Dual Drive USB C Memory Stick for Smartphone/Laptop/Tablet/PC - 128G, Blue</t>
+  </si>
+  <si>
+    <t>Display Port to HDMI Adapter</t>
+  </si>
+  <si>
+    <t>Amazon.com: UANTIN Display Port to HDMI 4K Adapter | Braided DP DisplayPort Male to HDMI Female Uni-Directional Converter for PC Dell HP AMD NVIDIA Laptop HDTV Monitor and Other Passive : Electronics</t>
+  </si>
+  <si>
+    <t>Display Port to HDMI 4K Adapter</t>
+  </si>
+  <si>
+    <t>Display Port to HDMI 4K Adapter | Braided DP DisplayPort Male to HDMI Female Uni-Directional Converter for PC Dell HP AMD NVIDIA Laptop HDTV Monitor and Other Passive</t>
+  </si>
+  <si>
+    <t>B0CYHB956B</t>
+  </si>
+  <si>
+    <t>USB female to USB C male adapter</t>
+  </si>
+  <si>
+    <t>B0DY5RJGCR</t>
+  </si>
+  <si>
+    <t>USB C to USB Adapter 4 Pack</t>
+  </si>
+  <si>
+    <t>Amazon.com: AVMAX USB C to USB Adapter 4 Pack,USBC Male to USB 3.0 Female OTG Adapter,Type C Male to A Female 3.0 OTG Adapter for Apple iPhone 16 15,Flash Thumb Drive,Mac,iPad,Samsung Galaxy : Electronics</t>
+  </si>
+  <si>
+    <t>AVMAX USB C to USB Adapter 4 Pack,USBC Male to USB 3.0 Female OTG Adapter,Type C Male to A Female 3.0 OTG Adapter for Apple iPhone 16 15,Flash Thumb Drive,Mac,iPad,Samsung Galaxy</t>
   </si>
 </sst>
 </file>
@@ -699,6 +759,12 @@
     <xf numFmtId="14" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -735,14 +801,8 @@
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1229,21 +1289,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3B39B8B-F33B-1140-8548-5838830ED406}">
   <dimension ref="B1:V37"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="31" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.125" bestFit="1" customWidth="1"/>
     <col min="7" max="9" width="16.5" customWidth="1"/>
-    <col min="11" max="11" width="12.1640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="24.83203125" customWidth="1"/>
+    <col min="11" max="11" width="12.125" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="24.875" customWidth="1"/>
     <col min="17" max="17" width="46.5" customWidth="1"/>
-    <col min="19" max="19" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="25.6640625" customWidth="1"/>
-    <col min="22" max="22" width="33.1640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="25.625" customWidth="1"/>
+    <col min="22" max="22" width="33.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:22" ht="29" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:22" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1292,13 +1352,13 @@
       <c r="Q2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="S2" s="45" t="s">
+      <c r="S2" s="47" t="s">
         <v>20</v>
       </c>
-      <c r="T2" s="45"/>
+      <c r="T2" s="47"/>
       <c r="U2" s="7"/>
     </row>
-    <row r="3" spans="2:22" ht="61" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:22" ht="60.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B3" s="39" t="s">
         <v>31</v>
       </c>
@@ -1316,12 +1376,14 @@
         <v>268.3</v>
       </c>
       <c r="G3" s="16" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="H3" s="34">
         <v>46201</v>
       </c>
-      <c r="I3" s="29"/>
+      <c r="I3" s="34">
+        <v>46209</v>
+      </c>
       <c r="J3" s="29" t="s">
         <v>38</v>
       </c>
@@ -1352,7 +1414,7 @@
       </c>
       <c r="U3" s="7"/>
     </row>
-    <row r="4" spans="2:22" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:22" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="39" t="s">
         <v>37</v>
       </c>
@@ -1384,7 +1446,7 @@
         <v>35</v>
       </c>
       <c r="M4" s="17"/>
-      <c r="N4" s="57" t="s">
+      <c r="N4" s="44" t="s">
         <v>36</v>
       </c>
       <c r="O4" s="24" t="s">
@@ -1400,7 +1462,7 @@
       <c r="T4" s="7"/>
       <c r="U4" s="7"/>
     </row>
-    <row r="5" spans="2:22" ht="75" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:22" ht="75" x14ac:dyDescent="0.25">
       <c r="B5" s="40" t="s">
         <v>59</v>
       </c>
@@ -1440,13 +1502,13 @@
       <c r="Q5" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="S5" s="46" t="s">
+      <c r="S5" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="T5" s="46"/>
+      <c r="T5" s="48"/>
       <c r="U5" s="7"/>
     </row>
-    <row r="6" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B6" s="39" t="s">
         <v>61</v>
       </c>
@@ -1474,13 +1536,13 @@
       <c r="O6" s="23"/>
       <c r="P6" s="36"/>
       <c r="Q6" s="32"/>
-      <c r="S6" s="43" t="s">
+      <c r="S6" s="45" t="s">
         <v>60</v>
       </c>
-      <c r="T6" s="43"/>
+      <c r="T6" s="45"/>
       <c r="U6" s="7"/>
     </row>
-    <row r="7" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B7" s="39" t="s">
         <v>62</v>
       </c>
@@ -1508,14 +1570,14 @@
       <c r="O7" s="23"/>
       <c r="P7" s="36"/>
       <c r="Q7" s="32"/>
-      <c r="S7" s="47" t="s">
+      <c r="S7" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="T7" s="47"/>
+      <c r="T7" s="49"/>
       <c r="U7" s="7"/>
     </row>
-    <row r="8" spans="2:22" ht="60" x14ac:dyDescent="0.2">
-      <c r="B8" s="55" t="s">
+    <row r="8" spans="2:22" ht="60" x14ac:dyDescent="0.25">
+      <c r="B8" s="5" t="s">
         <v>63</v>
       </c>
       <c r="C8" s="17">
@@ -1532,12 +1594,14 @@
         <v>48.48</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="H8" s="42">
         <v>46206</v>
       </c>
-      <c r="I8" s="30"/>
+      <c r="I8" s="57">
+        <v>46207</v>
+      </c>
       <c r="J8" s="30" t="s">
         <v>18</v>
       </c>
@@ -1548,10 +1612,10 @@
         <v>65</v>
       </c>
       <c r="M8" s="17"/>
-      <c r="N8" s="57" t="s">
+      <c r="N8" s="44" t="s">
         <v>68</v>
       </c>
-      <c r="O8" s="56" t="s">
+      <c r="O8" s="43" t="s">
         <v>67</v>
       </c>
       <c r="P8" s="37" t="s">
@@ -1560,121 +1624,229 @@
       <c r="Q8" s="31" t="s">
         <v>66</v>
       </c>
-      <c r="S8" s="48" t="s">
+      <c r="S8" s="50" t="s">
         <v>19</v>
       </c>
-      <c r="T8" s="48"/>
+      <c r="T8" s="50"/>
       <c r="U8" s="7"/>
     </row>
-    <row r="9" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="C9" s="16"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="18"/>
-      <c r="F9" s="19" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+    <row r="9" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B9" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C9" s="16">
+        <v>1</v>
+      </c>
+      <c r="D9" s="17">
+        <v>3</v>
+      </c>
+      <c r="E9" s="18">
+        <f>13.73/3</f>
+        <v>4.5766666666666671</v>
+      </c>
+      <c r="F9" s="19">
+        <f t="shared" si="0"/>
+        <v>13.73</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="H9" s="42"/>
+        <v>23</v>
+      </c>
+      <c r="H9" s="42">
+        <v>46209</v>
+      </c>
       <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17"/>
+      <c r="J9" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="K9" s="17" t="s">
+        <v>74</v>
+      </c>
       <c r="L9" s="17"/>
       <c r="M9" s="17"/>
-      <c r="N9" s="5"/>
-      <c r="O9" s="23"/>
-      <c r="P9" s="36"/>
-      <c r="Q9" s="32"/>
-      <c r="S9" s="49" t="s">
+      <c r="N9" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="O9" s="24" t="s">
+        <v>72</v>
+      </c>
+      <c r="P9" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q9" s="32" t="s">
+        <v>70</v>
+      </c>
+      <c r="R9" t="s">
+        <v>15</v>
+      </c>
+      <c r="S9" s="51" t="s">
         <v>23</v>
       </c>
-      <c r="T9" s="49"/>
+      <c r="T9" s="51"/>
       <c r="U9" s="7"/>
     </row>
-    <row r="10" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="19" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+    <row r="10" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B10" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C10" s="17">
+        <v>1</v>
+      </c>
+      <c r="D10" s="17">
+        <v>1</v>
+      </c>
+      <c r="E10" s="18">
+        <f>17.13-5.21+2.49</f>
+        <v>14.409999999999998</v>
+      </c>
+      <c r="F10" s="19">
+        <f t="shared" si="0"/>
+        <v>14.409999999999998</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="H10" s="42"/>
+        <v>23</v>
+      </c>
+      <c r="H10" s="42">
+        <v>46209</v>
+      </c>
       <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="17"/>
+      <c r="J10" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="K10" s="17" t="s">
+        <v>75</v>
+      </c>
       <c r="L10" s="17"/>
       <c r="M10" s="17"/>
-      <c r="N10" s="5"/>
-      <c r="O10" s="23"/>
-      <c r="P10" s="36"/>
-      <c r="Q10" s="32"/>
-      <c r="S10" s="50" t="s">
+      <c r="N10" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="O10" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="P10" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q10" s="32" t="s">
+        <v>78</v>
+      </c>
+      <c r="R10" t="s">
+        <v>15</v>
+      </c>
+      <c r="S10" s="52" t="s">
         <v>24</v>
       </c>
-      <c r="T10" s="50"/>
+      <c r="T10" s="52"/>
       <c r="U10" s="7"/>
     </row>
-    <row r="11" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="C11" s="16"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="19" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+    <row r="11" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B11" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C11" s="16">
+        <v>1</v>
+      </c>
+      <c r="D11" s="17">
+        <v>1</v>
+      </c>
+      <c r="E11" s="18">
+        <v>7.99</v>
+      </c>
+      <c r="F11" s="19">
+        <f t="shared" si="0"/>
+        <v>7.99</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="H11" s="42"/>
+        <v>23</v>
+      </c>
+      <c r="H11" s="42">
+        <v>46209</v>
+      </c>
       <c r="I11" s="17"/>
-      <c r="J11" s="17"/>
-      <c r="K11" s="17"/>
+      <c r="J11" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="K11" s="17" t="s">
+        <v>83</v>
+      </c>
       <c r="L11" s="17"/>
       <c r="M11" s="17"/>
-      <c r="N11" s="5"/>
-      <c r="O11" s="23"/>
-      <c r="P11" s="36"/>
-      <c r="Q11" s="32"/>
-      <c r="S11" s="51" t="s">
+      <c r="N11" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="O11" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="P11" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q11" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="R11" t="s">
+        <v>15</v>
+      </c>
+      <c r="S11" s="53" t="s">
         <v>25</v>
       </c>
-      <c r="T11" s="51"/>
+      <c r="T11" s="53"/>
       <c r="U11" s="7"/>
     </row>
-    <row r="12" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="19" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+    <row r="12" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B12" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C12" s="17">
+        <v>1</v>
+      </c>
+      <c r="D12" s="17">
+        <v>4</v>
+      </c>
+      <c r="E12" s="18">
+        <f>6.99/4</f>
+        <v>1.7475000000000001</v>
+      </c>
+      <c r="F12" s="19">
+        <f t="shared" si="0"/>
+        <v>6.99</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="H12" s="42"/>
+        <v>23</v>
+      </c>
+      <c r="H12" s="42">
+        <v>46209</v>
+      </c>
       <c r="I12" s="17"/>
-      <c r="J12" s="17"/>
-      <c r="K12" s="17"/>
+      <c r="J12" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="K12" s="17" t="s">
+        <v>85</v>
+      </c>
       <c r="L12" s="17"/>
       <c r="M12" s="17"/>
-      <c r="N12" s="5"/>
-      <c r="O12" s="23"/>
-      <c r="P12" s="36"/>
-      <c r="Q12" s="32"/>
-      <c r="S12" s="52" t="s">
+      <c r="N12" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="O12" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="P12" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q12" s="32" t="s">
+        <v>88</v>
+      </c>
+      <c r="R12" t="s">
+        <v>15</v>
+      </c>
+      <c r="S12" s="54" t="s">
         <v>26</v>
       </c>
-      <c r="T12" s="52"/>
+      <c r="T12" s="54"/>
       <c r="U12" s="7"/>
     </row>
-    <row r="13" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B13" s="5"/>
       <c r="C13" s="17"/>
       <c r="D13" s="17"/>
       <c r="E13" s="18"/>
@@ -1695,13 +1867,14 @@
       <c r="O13" s="20"/>
       <c r="P13" s="35"/>
       <c r="Q13" s="32"/>
-      <c r="S13" s="53" t="s">
+      <c r="S13" s="55" t="s">
         <v>27</v>
       </c>
-      <c r="T13" s="53"/>
+      <c r="T13" s="55"/>
       <c r="U13" s="7"/>
     </row>
-    <row r="14" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B14" s="5"/>
       <c r="C14" s="16"/>
       <c r="D14" s="17"/>
       <c r="E14" s="18"/>
@@ -1722,13 +1895,14 @@
       <c r="O14" s="23"/>
       <c r="P14" s="36"/>
       <c r="Q14" s="32"/>
-      <c r="S14" s="54" t="s">
+      <c r="S14" s="56" t="s">
         <v>16</v>
       </c>
-      <c r="T14" s="54"/>
+      <c r="T14" s="56"/>
       <c r="U14" s="7"/>
     </row>
-    <row r="15" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B15" s="5"/>
       <c r="C15" s="17"/>
       <c r="D15" s="17"/>
       <c r="E15" s="18"/>
@@ -1749,13 +1923,14 @@
       <c r="O15" s="24"/>
       <c r="P15" s="22"/>
       <c r="Q15" s="32"/>
-      <c r="S15" s="44" t="s">
+      <c r="S15" s="46" t="s">
         <v>14</v>
       </c>
-      <c r="T15" s="44"/>
+      <c r="T15" s="46"/>
       <c r="U15" s="7"/>
     </row>
-    <row r="16" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B16" s="5"/>
       <c r="C16" s="17"/>
       <c r="D16" s="17"/>
       <c r="E16" s="18"/>
@@ -1779,7 +1954,8 @@
       <c r="U16" s="7"/>
       <c r="V16" s="7"/>
     </row>
-    <row r="17" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B17" s="5"/>
       <c r="C17" s="16"/>
       <c r="D17" s="17"/>
       <c r="E17" s="18"/>
@@ -1803,7 +1979,8 @@
       <c r="S17" s="7"/>
       <c r="V17" s="7"/>
     </row>
-    <row r="18" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B18" s="5"/>
       <c r="C18" s="17"/>
       <c r="D18" s="17"/>
       <c r="E18" s="18"/>
@@ -1827,8 +2004,8 @@
       <c r="S18" s="7"/>
       <c r="V18" s="7"/>
     </row>
-    <row r="19" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B19" s="39" t="s">
+    <row r="19" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B19" s="5" t="s">
         <v>42</v>
       </c>
       <c r="C19" s="16"/>
@@ -1854,8 +2031,8 @@
       <c r="S19" s="7"/>
       <c r="V19" s="7"/>
     </row>
-    <row r="20" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B20" s="39" t="s">
+    <row r="20" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B20" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C20" s="16"/>
@@ -1881,8 +2058,8 @@
       <c r="S20" s="7"/>
       <c r="V20" s="7"/>
     </row>
-    <row r="21" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B21" s="39" t="s">
+    <row r="21" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B21" s="5" t="s">
         <v>44</v>
       </c>
       <c r="C21" s="17"/>
@@ -1906,7 +2083,7 @@
       <c r="P21" s="35"/>
       <c r="Q21" s="32"/>
     </row>
-    <row r="22" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B22" s="39" t="s">
         <v>45</v>
       </c>
@@ -1931,7 +2108,7 @@
       <c r="P22" s="36"/>
       <c r="Q22" s="32"/>
     </row>
-    <row r="23" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="39" t="s">
         <v>46</v>
       </c>
@@ -1956,7 +2133,7 @@
       <c r="P23" s="35"/>
       <c r="Q23" s="32"/>
     </row>
-    <row r="24" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B24" s="39" t="s">
         <v>47</v>
       </c>
@@ -1987,7 +2164,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="25" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B25" s="39" t="s">
         <v>48</v>
       </c>
@@ -2016,10 +2193,10 @@
       </c>
       <c r="T25" s="13">
         <f>SUM(F3:F37)</f>
-        <v>341.77000000000004</v>
-      </c>
-    </row>
-    <row r="26" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+        <v>384.8900000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="2:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="39" t="s">
         <v>49</v>
       </c>
@@ -2048,10 +2225,10 @@
       </c>
       <c r="T26" s="15">
         <f>T24-T25</f>
-        <v>1658.23</v>
-      </c>
-    </row>
-    <row r="27" spans="2:22" x14ac:dyDescent="0.2">
+        <v>1615.11</v>
+      </c>
+    </row>
+    <row r="27" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B27" s="39" t="s">
         <v>50</v>
       </c>
@@ -2076,7 +2253,7 @@
       <c r="P27" s="35"/>
       <c r="Q27" s="32"/>
     </row>
-    <row r="28" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B28" s="39" t="s">
         <v>51</v>
       </c>
@@ -2101,7 +2278,7 @@
       <c r="P28" s="36"/>
       <c r="Q28" s="32"/>
     </row>
-    <row r="29" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B29" s="39" t="s">
         <v>52</v>
       </c>
@@ -2126,7 +2303,7 @@
       <c r="P29" s="36"/>
       <c r="Q29" s="32"/>
     </row>
-    <row r="30" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B30" s="39"/>
       <c r="C30" s="16"/>
       <c r="D30" s="17"/>
@@ -2149,7 +2326,7 @@
       <c r="P30" s="36"/>
       <c r="Q30" s="32"/>
     </row>
-    <row r="31" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B31" s="39"/>
       <c r="C31" s="17"/>
       <c r="D31" s="17"/>
@@ -2172,7 +2349,7 @@
       <c r="P31" s="36"/>
       <c r="Q31" s="32"/>
     </row>
-    <row r="32" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B32" s="39"/>
       <c r="C32" s="17"/>
       <c r="D32" s="17"/>
@@ -2195,7 +2372,7 @@
       <c r="P32" s="36"/>
       <c r="Q32" s="32"/>
     </row>
-    <row r="33" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B33" s="39"/>
       <c r="C33" s="16"/>
       <c r="D33" s="17"/>
@@ -2218,7 +2395,7 @@
       <c r="P33" s="36"/>
       <c r="Q33" s="32"/>
     </row>
-    <row r="34" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B34" s="39"/>
       <c r="C34" s="17"/>
       <c r="D34" s="17"/>
@@ -2241,7 +2418,7 @@
       <c r="P34" s="36"/>
       <c r="Q34" s="32"/>
     </row>
-    <row r="35" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B35" s="39"/>
       <c r="C35" s="17"/>
       <c r="D35" s="17"/>
@@ -2264,7 +2441,7 @@
       <c r="P35" s="36"/>
       <c r="Q35" s="32"/>
     </row>
-    <row r="36" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B36" s="39"/>
       <c r="C36" s="17"/>
       <c r="D36" s="17"/>
@@ -2287,7 +2464,7 @@
       <c r="P36" s="36"/>
       <c r="Q36" s="32"/>
     </row>
-    <row r="37" spans="2:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B37" s="41"/>
       <c r="C37" s="25"/>
       <c r="D37" s="25"/>
@@ -2398,6 +2575,7 @@
     <hyperlink ref="P5" r:id="rId4" xr:uid="{8F840528-6D9F-4456-8BB5-74A65BFEE351}"/>
     <hyperlink ref="O5" r:id="rId5" display="https://vilros.com/products/vilros-soldering-iron-kit-electronics-14-in-1-60w-adjustable-temperature-soldering-iron-with-on-off-switch-5pcs-soldering-iron-tips-desoldering-pump-tweezers-stand-solder-pu-carry-bag?variant=31184817684574&amp;country=US&amp;currency=USD&amp;utm_medium=product_sync&amp;utm_source=google&amp;utm_content=sag_organic&amp;utm_campaign=sag_organic&amp;tw_source=google&amp;tw_adid=&amp;tw_campaign=18070425970&amp;gad_source=1&amp;gad_campaignid=17177576781&amp;gbraid=0AAAAAD1QJAhpwOz4TG9imhRizOjsiF33r&amp;gclid=Cj0KCQjwr4jSBhCSARIsAOX1E-IcDf7VArvc12fU96XQu_eogR6Cku3p0W322S9UE6enAxh-gCdhcRkaApEYEALw_wcB" xr:uid="{F8EE24A7-3DF2-4835-8818-4CF5FD2EFD11}"/>
     <hyperlink ref="O8" r:id="rId6" xr:uid="{ED02DEDC-B0EC-0749-B7B9-A7D73B4129EF}"/>
+    <hyperlink ref="O9" r:id="rId7" xr:uid="{5B52362B-868D-40C8-ADAC-0C067B706503}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
wifi and STM BOM update
</commit_message>
<xml_diff>
--- a/docs/financials/Buddy_BOM.xlsx
+++ b/docs/financials/Buddy_BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\venti\Desktop\Buddy_Robot\docs\financials\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ventimaj/Desktop/Desktop - MacBook Air (263)/Buddy_Robot/docs/financials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6010315A-D91F-48F0-9EB4-4B1A3CAF49B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DA2F662-2898-A243-8BCD-A3C5B8DC8AB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{C64966AC-B3BB-9844-956C-858996BC28CC}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17420" xr2:uid="{C64966AC-B3BB-9844-956C-858996BC28CC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="96">
   <si>
     <t>Descriptive Part Name</t>
   </si>
@@ -190,12 +190,6 @@
     <t>E-Stop Button</t>
   </si>
   <si>
-    <t>ESP or STM or Teensy</t>
-  </si>
-  <si>
-    <t>Power supply</t>
-  </si>
-  <si>
     <t>Oscilloscope</t>
   </si>
   <si>
@@ -308,6 +302,33 @@
   </si>
   <si>
     <t>AVMAX USB C to USB Adapter 4 Pack,USBC Male to USB 3.0 Female OTG Adapter,Type C Male to A Female 3.0 OTG Adapter for Apple iPhone 16 15,Flash Thumb Drive,Mac,iPad,Samsung Galaxy</t>
+  </si>
+  <si>
+    <t>NUCLEO-G474RE</t>
+  </si>
+  <si>
+    <t>STMelectronics</t>
+  </si>
+  <si>
+    <t>UPS GROUND: 1Z7759450324444260</t>
+  </si>
+  <si>
+    <t>TP-Link Deco AXE5400 Tri-Band WiFi 6E Mesh System(Deco XE75)</t>
+  </si>
+  <si>
+    <t>Best Buy</t>
+  </si>
+  <si>
+    <t>TP-Link - Deco XE75 Pro AXE5400 Tri-Band Wi-Fi 6E Whole Home Mesh System (3-Pack) - White</t>
+  </si>
+  <si>
+    <t>https://www.bestbuy.com/product/tp-link-deco-xe75-pro-axe5400-tri-band-wi-fi-6e-whole-home-mesh-system-3-pack-white/J39QK2QCVK/sku/6508223?utm_source=feed&amp;extStoreId=111&amp;ref=212&amp;loc=19617835341&amp;gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=19625924345&amp;gbraid=0AAAAAD-ORIgcydh608nRdNrV3WhPxnAlz&amp;gclid=CjwKCAjwpqHTBhAcEiwAj2Afuo2MoewbEOvsHoLL6QQb_ILA0lsz_piC7A98Ldy_NmqzwlrjcYsPlxoCIAYQAvD_BwE</t>
+  </si>
+  <si>
+    <t>SKU: 6508223</t>
+  </si>
+  <si>
+    <t>Tri-band</t>
   </si>
 </sst>
 </file>
@@ -765,6 +786,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -800,9 +824,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1289,21 +1310,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3B39B8B-F33B-1140-8548-5838830ED406}">
   <dimension ref="B1:V37"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="31" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="9" width="16.5" customWidth="1"/>
-    <col min="11" max="11" width="12.125" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="24.875" customWidth="1"/>
+    <col min="10" max="11" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="15" max="16" width="24.83203125" customWidth="1"/>
     <col min="17" max="17" width="46.5" customWidth="1"/>
-    <col min="19" max="19" width="12.375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="25.625" customWidth="1"/>
-    <col min="22" max="22" width="33.125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="25.6640625" customWidth="1"/>
+    <col min="22" max="22" width="33.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:22" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:22" ht="29" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1323,10 +1344,10 @@
         <v>5</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>6</v>
@@ -1347,18 +1368,18 @@
         <v>11</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="Q2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="S2" s="47" t="s">
+      <c r="S2" s="48" t="s">
         <v>20</v>
       </c>
-      <c r="T2" s="47"/>
+      <c r="T2" s="48"/>
       <c r="U2" s="7"/>
     </row>
-    <row r="3" spans="2:22" ht="60.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:22" ht="61" thickTop="1" x14ac:dyDescent="0.2">
       <c r="B3" s="39" t="s">
         <v>31</v>
       </c>
@@ -1403,7 +1424,7 @@
         <v>40</v>
       </c>
       <c r="P3" s="22" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="Q3" s="31" t="s">
         <v>41</v>
@@ -1414,7 +1435,7 @@
       </c>
       <c r="U3" s="7"/>
     </row>
-    <row r="4" spans="2:22" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:22" ht="60" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="39" t="s">
         <v>37</v>
       </c>
@@ -1432,7 +1453,7 @@
         <v/>
       </c>
       <c r="G4" s="16" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="H4" s="29"/>
       <c r="I4" s="29"/>
@@ -1462,9 +1483,9 @@
       <c r="T4" s="7"/>
       <c r="U4" s="7"/>
     </row>
-    <row r="5" spans="2:22" ht="75" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:22" ht="75" x14ac:dyDescent="0.2">
       <c r="B5" s="40" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C5" s="16">
         <v>1</v>
@@ -1494,23 +1515,23 @@
       <c r="M5" s="17"/>
       <c r="N5" s="5"/>
       <c r="O5" s="24" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="P5" s="22" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="Q5" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="S5" s="48" t="s">
+      <c r="S5" s="49" t="s">
         <v>21</v>
       </c>
-      <c r="T5" s="48"/>
+      <c r="T5" s="49"/>
       <c r="U5" s="7"/>
     </row>
-    <row r="6" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B6" s="39" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C6" s="17">
         <v>1</v>
@@ -1524,7 +1545,7 @@
         <v/>
       </c>
       <c r="G6" s="16" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H6" s="42"/>
       <c r="I6" s="17"/>
@@ -1536,15 +1557,15 @@
       <c r="O6" s="23"/>
       <c r="P6" s="36"/>
       <c r="Q6" s="32"/>
-      <c r="S6" s="45" t="s">
+      <c r="S6" s="46" t="s">
+        <v>58</v>
+      </c>
+      <c r="T6" s="46"/>
+      <c r="U6" s="7"/>
+    </row>
+    <row r="7" spans="2:22" x14ac:dyDescent="0.2">
+      <c r="B7" s="39" t="s">
         <v>60</v>
-      </c>
-      <c r="T6" s="45"/>
-      <c r="U6" s="7"/>
-    </row>
-    <row r="7" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B7" s="39" t="s">
-        <v>62</v>
       </c>
       <c r="C7" s="16">
         <v>1</v>
@@ -1558,7 +1579,7 @@
         <v/>
       </c>
       <c r="G7" s="16" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="H7" s="42"/>
       <c r="I7" s="17"/>
@@ -1570,15 +1591,15 @@
       <c r="O7" s="23"/>
       <c r="P7" s="36"/>
       <c r="Q7" s="32"/>
-      <c r="S7" s="49" t="s">
+      <c r="S7" s="50" t="s">
         <v>17</v>
       </c>
-      <c r="T7" s="49"/>
+      <c r="T7" s="50"/>
       <c r="U7" s="7"/>
     </row>
-    <row r="8" spans="2:22" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:22" ht="60" x14ac:dyDescent="0.2">
       <c r="B8" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C8" s="17">
         <v>1</v>
@@ -1599,40 +1620,40 @@
       <c r="H8" s="42">
         <v>46206</v>
       </c>
-      <c r="I8" s="57">
+      <c r="I8" s="45">
         <v>46207</v>
       </c>
       <c r="J8" s="30" t="s">
         <v>18</v>
       </c>
       <c r="K8" s="17" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="L8" s="17" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="M8" s="17"/>
       <c r="N8" s="44" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O8" s="43" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="P8" s="37" t="s">
         <v>15</v>
       </c>
       <c r="Q8" s="31" t="s">
-        <v>66</v>
-      </c>
-      <c r="S8" s="50" t="s">
+        <v>64</v>
+      </c>
+      <c r="S8" s="51" t="s">
         <v>19</v>
       </c>
-      <c r="T8" s="50"/>
+      <c r="T8" s="51"/>
       <c r="U8" s="7"/>
     </row>
-    <row r="9" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B9" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C9" s="16">
         <v>1</v>
@@ -1649,44 +1670,44 @@
         <v>13.73</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="H9" s="42">
         <v>46209</v>
       </c>
-      <c r="I9" s="17"/>
+      <c r="I9" s="45"/>
       <c r="J9" s="17" t="s">
         <v>18</v>
       </c>
       <c r="K9" s="17" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="L9" s="17"/>
       <c r="M9" s="17"/>
       <c r="N9" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O9" s="24" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="P9" s="36" t="s">
         <v>15</v>
       </c>
       <c r="Q9" s="32" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="R9" t="s">
         <v>15</v>
       </c>
-      <c r="S9" s="51" t="s">
+      <c r="S9" s="52" t="s">
         <v>23</v>
       </c>
-      <c r="T9" s="51"/>
+      <c r="T9" s="52"/>
       <c r="U9" s="7"/>
     </row>
-    <row r="10" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B10" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C10" s="17">
         <v>1</v>
@@ -1703,44 +1724,44 @@
         <v>14.409999999999998</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="H10" s="42">
         <v>46209</v>
       </c>
-      <c r="I10" s="17"/>
+      <c r="I10" s="45"/>
       <c r="J10" s="17" t="s">
         <v>18</v>
       </c>
       <c r="K10" s="17" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="L10" s="17"/>
       <c r="M10" s="17"/>
       <c r="N10" s="5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="O10" s="23" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="P10" s="36" t="s">
         <v>15</v>
       </c>
       <c r="Q10" s="32" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="R10" t="s">
         <v>15</v>
       </c>
-      <c r="S10" s="52" t="s">
+      <c r="S10" s="53" t="s">
         <v>24</v>
       </c>
-      <c r="T10" s="52"/>
+      <c r="T10" s="53"/>
       <c r="U10" s="7"/>
     </row>
-    <row r="11" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B11" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C11" s="16">
         <v>1</v>
@@ -1756,44 +1777,44 @@
         <v>7.99</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="H11" s="42">
         <v>46209</v>
       </c>
-      <c r="I11" s="17"/>
+      <c r="I11" s="45"/>
       <c r="J11" s="17" t="s">
         <v>18</v>
       </c>
       <c r="K11" s="17" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L11" s="17"/>
       <c r="M11" s="17"/>
       <c r="N11" s="5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="O11" s="23" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="P11" s="36" t="s">
         <v>15</v>
       </c>
       <c r="Q11" s="32" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="R11" t="s">
         <v>15</v>
       </c>
-      <c r="S11" s="53" t="s">
+      <c r="S11" s="54" t="s">
         <v>25</v>
       </c>
-      <c r="T11" s="53"/>
+      <c r="T11" s="54"/>
       <c r="U11" s="7"/>
     </row>
-    <row r="12" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B12" s="5" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C12" s="17">
         <v>1</v>
@@ -1810,98 +1831,137 @@
         <v>6.99</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="H12" s="42">
         <v>46209</v>
       </c>
-      <c r="I12" s="17"/>
+      <c r="I12" s="45"/>
       <c r="J12" s="17" t="s">
         <v>18</v>
       </c>
       <c r="K12" s="17" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L12" s="17"/>
       <c r="M12" s="17"/>
       <c r="N12" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="O12" s="23" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="P12" s="36" t="s">
         <v>15</v>
       </c>
       <c r="Q12" s="32" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="R12" t="s">
         <v>15</v>
       </c>
-      <c r="S12" s="54" t="s">
+      <c r="S12" s="55" t="s">
         <v>26</v>
       </c>
-      <c r="T12" s="54"/>
+      <c r="T12" s="55"/>
       <c r="U12" s="7"/>
     </row>
-    <row r="13" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B13" s="5"/>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="19" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+    <row r="13" spans="2:22" x14ac:dyDescent="0.2">
+      <c r="B13" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C13" s="17">
+        <v>1</v>
+      </c>
+      <c r="D13" s="17">
+        <v>2</v>
+      </c>
+      <c r="E13" s="18">
+        <f>48.97/2</f>
+        <v>24.484999999999999</v>
+      </c>
+      <c r="F13" s="19">
+        <f t="shared" si="0"/>
+        <v>48.97</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="H13" s="42"/>
-      <c r="I13" s="29"/>
-      <c r="J13" s="29"/>
+        <v>23</v>
+      </c>
+      <c r="H13" s="42">
+        <v>46228</v>
+      </c>
+      <c r="I13" s="45"/>
+      <c r="J13" s="29" t="s">
+        <v>88</v>
+      </c>
       <c r="K13" s="17"/>
       <c r="L13" s="17"/>
       <c r="M13" s="17"/>
       <c r="N13" s="5"/>
       <c r="O13" s="20"/>
-      <c r="P13" s="35"/>
+      <c r="P13" s="32" t="s">
+        <v>89</v>
+      </c>
       <c r="Q13" s="32"/>
-      <c r="S13" s="55" t="s">
+      <c r="S13" s="56" t="s">
         <v>27</v>
       </c>
-      <c r="T13" s="55"/>
+      <c r="T13" s="56"/>
       <c r="U13" s="7"/>
     </row>
-    <row r="14" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B14" s="5"/>
-      <c r="C14" s="16"/>
-      <c r="D14" s="17"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="19" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+    <row r="14" spans="2:22" x14ac:dyDescent="0.2">
+      <c r="B14" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C14" s="16">
+        <v>1</v>
+      </c>
+      <c r="D14" s="17">
+        <v>1</v>
+      </c>
+      <c r="E14" s="18">
+        <v>294.95999999999998</v>
+      </c>
+      <c r="F14" s="19">
+        <f t="shared" si="0"/>
+        <v>294.95999999999998</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="H14" s="42"/>
-      <c r="I14" s="17"/>
-      <c r="J14" s="17"/>
-      <c r="K14" s="17"/>
+        <v>17</v>
+      </c>
+      <c r="H14" s="42">
+        <v>46231</v>
+      </c>
+      <c r="I14" s="45">
+        <v>46231</v>
+      </c>
+      <c r="J14" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="K14" s="17" t="s">
+        <v>94</v>
+      </c>
       <c r="L14" s="17"/>
       <c r="M14" s="17"/>
-      <c r="N14" s="5"/>
-      <c r="O14" s="23"/>
-      <c r="P14" s="36"/>
-      <c r="Q14" s="32"/>
-      <c r="S14" s="56" t="s">
+      <c r="N14" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="O14" s="23" t="s">
+        <v>93</v>
+      </c>
+      <c r="P14" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q14" s="32" t="s">
+        <v>92</v>
+      </c>
+      <c r="S14" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="T14" s="56"/>
+      <c r="T14" s="57"/>
       <c r="U14" s="7"/>
     </row>
-    <row r="15" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B15" s="5"/>
       <c r="C15" s="17"/>
       <c r="D15" s="17"/>
@@ -1914,7 +1974,7 @@
         <v>14</v>
       </c>
       <c r="H15" s="42"/>
-      <c r="I15" s="17"/>
+      <c r="I15" s="45"/>
       <c r="J15" s="17"/>
       <c r="K15" s="17"/>
       <c r="L15" s="17"/>
@@ -1923,13 +1983,13 @@
       <c r="O15" s="24"/>
       <c r="P15" s="22"/>
       <c r="Q15" s="32"/>
-      <c r="S15" s="46" t="s">
+      <c r="S15" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="T15" s="46"/>
+      <c r="T15" s="47"/>
       <c r="U15" s="7"/>
     </row>
-    <row r="16" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B16" s="5"/>
       <c r="C16" s="17"/>
       <c r="D16" s="17"/>
@@ -1942,7 +2002,7 @@
         <v>14</v>
       </c>
       <c r="H16" s="42"/>
-      <c r="I16" s="29"/>
+      <c r="I16" s="45"/>
       <c r="J16" s="29"/>
       <c r="K16" s="17"/>
       <c r="L16" s="17"/>
@@ -1954,7 +2014,7 @@
       <c r="U16" s="7"/>
       <c r="V16" s="7"/>
     </row>
-    <row r="17" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B17" s="5"/>
       <c r="C17" s="16"/>
       <c r="D17" s="17"/>
@@ -1967,7 +2027,7 @@
         <v>14</v>
       </c>
       <c r="H17" s="42"/>
-      <c r="I17" s="17"/>
+      <c r="I17" s="45"/>
       <c r="J17" s="17"/>
       <c r="K17" s="17"/>
       <c r="L17" s="17"/>
@@ -1979,7 +2039,7 @@
       <c r="S17" s="7"/>
       <c r="V17" s="7"/>
     </row>
-    <row r="18" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B18" s="5"/>
       <c r="C18" s="17"/>
       <c r="D18" s="17"/>
@@ -1992,7 +2052,7 @@
         <v>14</v>
       </c>
       <c r="H18" s="42"/>
-      <c r="I18" s="17"/>
+      <c r="I18" s="45"/>
       <c r="J18" s="17"/>
       <c r="K18" s="17"/>
       <c r="L18" s="17"/>
@@ -2004,7 +2064,7 @@
       <c r="S18" s="7"/>
       <c r="V18" s="7"/>
     </row>
-    <row r="19" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B19" s="5" t="s">
         <v>42</v>
       </c>
@@ -2019,7 +2079,7 @@
         <v>14</v>
       </c>
       <c r="H19" s="42"/>
-      <c r="I19" s="17"/>
+      <c r="I19" s="45"/>
       <c r="J19" s="17"/>
       <c r="K19" s="17"/>
       <c r="L19" s="17"/>
@@ -2031,7 +2091,7 @@
       <c r="S19" s="7"/>
       <c r="V19" s="7"/>
     </row>
-    <row r="20" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B20" s="5" t="s">
         <v>43</v>
       </c>
@@ -2046,7 +2106,7 @@
         <v>14</v>
       </c>
       <c r="H20" s="42"/>
-      <c r="I20" s="29"/>
+      <c r="I20" s="45"/>
       <c r="J20" s="29"/>
       <c r="K20" s="17"/>
       <c r="L20" s="17"/>
@@ -2058,7 +2118,7 @@
       <c r="S20" s="7"/>
       <c r="V20" s="7"/>
     </row>
-    <row r="21" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B21" s="5" t="s">
         <v>44</v>
       </c>
@@ -2073,7 +2133,7 @@
         <v>14</v>
       </c>
       <c r="H21" s="29"/>
-      <c r="I21" s="29"/>
+      <c r="I21" s="45"/>
       <c r="J21" s="29"/>
       <c r="K21" s="17"/>
       <c r="L21" s="17"/>
@@ -2083,7 +2143,7 @@
       <c r="P21" s="35"/>
       <c r="Q21" s="32"/>
     </row>
-    <row r="22" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B22" s="39" t="s">
         <v>45</v>
       </c>
@@ -2098,7 +2158,7 @@
         <v>14</v>
       </c>
       <c r="H22" s="17"/>
-      <c r="I22" s="17"/>
+      <c r="I22" s="45"/>
       <c r="J22" s="17"/>
       <c r="K22" s="17"/>
       <c r="L22" s="17"/>
@@ -2108,7 +2168,7 @@
       <c r="P22" s="36"/>
       <c r="Q22" s="32"/>
     </row>
-    <row r="23" spans="2:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B23" s="39" t="s">
         <v>46</v>
       </c>
@@ -2123,7 +2183,7 @@
         <v>14</v>
       </c>
       <c r="H23" s="17"/>
-      <c r="I23" s="17"/>
+      <c r="I23" s="45"/>
       <c r="J23" s="17"/>
       <c r="K23" s="17"/>
       <c r="L23" s="17"/>
@@ -2133,7 +2193,7 @@
       <c r="P23" s="35"/>
       <c r="Q23" s="32"/>
     </row>
-    <row r="24" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B24" s="39" t="s">
         <v>47</v>
       </c>
@@ -2148,7 +2208,7 @@
         <v>14</v>
       </c>
       <c r="H24" s="17"/>
-      <c r="I24" s="17"/>
+      <c r="I24" s="45"/>
       <c r="J24" s="17"/>
       <c r="K24" s="17"/>
       <c r="L24" s="17"/>
@@ -2164,7 +2224,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="25" spans="2:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B25" s="39" t="s">
         <v>48</v>
       </c>
@@ -2179,7 +2239,7 @@
         <v>14</v>
       </c>
       <c r="H25" s="29"/>
-      <c r="I25" s="29"/>
+      <c r="I25" s="45"/>
       <c r="J25" s="29"/>
       <c r="K25" s="17"/>
       <c r="L25" s="17"/>
@@ -2193,13 +2253,11 @@
       </c>
       <c r="T25" s="13">
         <f>SUM(F3:F37)</f>
-        <v>384.8900000000001</v>
-      </c>
-    </row>
-    <row r="26" spans="2:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="39" t="s">
-        <v>49</v>
-      </c>
+        <v>728.82000000000016</v>
+      </c>
+    </row>
+    <row r="26" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="39"/>
       <c r="C26" s="16"/>
       <c r="D26" s="17"/>
       <c r="E26" s="18"/>
@@ -2211,7 +2269,7 @@
         <v>14</v>
       </c>
       <c r="H26" s="17"/>
-      <c r="I26" s="17"/>
+      <c r="I26" s="45"/>
       <c r="J26" s="17"/>
       <c r="K26" s="17"/>
       <c r="L26" s="17"/>
@@ -2225,13 +2283,11 @@
       </c>
       <c r="T26" s="15">
         <f>T24-T25</f>
-        <v>1615.11</v>
-      </c>
-    </row>
-    <row r="27" spans="2:22" x14ac:dyDescent="0.25">
-      <c r="B27" s="39" t="s">
-        <v>50</v>
-      </c>
+        <v>1271.1799999999998</v>
+      </c>
+    </row>
+    <row r="27" spans="2:22" x14ac:dyDescent="0.2">
+      <c r="B27" s="39"/>
       <c r="C27" s="17"/>
       <c r="D27" s="17"/>
       <c r="E27" s="18"/>
@@ -2243,7 +2299,7 @@
         <v>14</v>
       </c>
       <c r="H27" s="17"/>
-      <c r="I27" s="17"/>
+      <c r="I27" s="45"/>
       <c r="J27" s="17"/>
       <c r="K27" s="17"/>
       <c r="L27" s="17"/>
@@ -2253,9 +2309,9 @@
       <c r="P27" s="35"/>
       <c r="Q27" s="32"/>
     </row>
-    <row r="28" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B28" s="39" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C28" s="16"/>
       <c r="D28" s="17"/>
@@ -2268,7 +2324,7 @@
         <v>14</v>
       </c>
       <c r="H28" s="17"/>
-      <c r="I28" s="17"/>
+      <c r="I28" s="45"/>
       <c r="J28" s="17"/>
       <c r="K28" s="17"/>
       <c r="L28" s="17"/>
@@ -2278,9 +2334,9 @@
       <c r="P28" s="36"/>
       <c r="Q28" s="32"/>
     </row>
-    <row r="29" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B29" s="39" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C29" s="17"/>
       <c r="D29" s="17"/>
@@ -2293,7 +2349,7 @@
         <v>14</v>
       </c>
       <c r="H29" s="17"/>
-      <c r="I29" s="17"/>
+      <c r="I29" s="45"/>
       <c r="J29" s="17"/>
       <c r="K29" s="17"/>
       <c r="L29" s="17"/>
@@ -2303,7 +2359,7 @@
       <c r="P29" s="36"/>
       <c r="Q29" s="32"/>
     </row>
-    <row r="30" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B30" s="39"/>
       <c r="C30" s="16"/>
       <c r="D30" s="17"/>
@@ -2316,7 +2372,7 @@
         <v>14</v>
       </c>
       <c r="H30" s="17"/>
-      <c r="I30" s="17"/>
+      <c r="I30" s="45"/>
       <c r="J30" s="17"/>
       <c r="K30" s="17"/>
       <c r="L30" s="17"/>
@@ -2326,7 +2382,7 @@
       <c r="P30" s="36"/>
       <c r="Q30" s="32"/>
     </row>
-    <row r="31" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B31" s="39"/>
       <c r="C31" s="17"/>
       <c r="D31" s="17"/>
@@ -2339,7 +2395,7 @@
         <v>14</v>
       </c>
       <c r="H31" s="17"/>
-      <c r="I31" s="17"/>
+      <c r="I31" s="45"/>
       <c r="J31" s="17"/>
       <c r="K31" s="17"/>
       <c r="L31" s="17"/>
@@ -2349,7 +2405,7 @@
       <c r="P31" s="36"/>
       <c r="Q31" s="32"/>
     </row>
-    <row r="32" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:22" x14ac:dyDescent="0.2">
       <c r="B32" s="39"/>
       <c r="C32" s="17"/>
       <c r="D32" s="17"/>
@@ -2362,7 +2418,7 @@
         <v>14</v>
       </c>
       <c r="H32" s="17"/>
-      <c r="I32" s="17"/>
+      <c r="I32" s="45"/>
       <c r="J32" s="17"/>
       <c r="K32" s="17"/>
       <c r="L32" s="17"/>
@@ -2372,7 +2428,7 @@
       <c r="P32" s="36"/>
       <c r="Q32" s="32"/>
     </row>
-    <row r="33" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B33" s="39"/>
       <c r="C33" s="16"/>
       <c r="D33" s="17"/>
@@ -2385,7 +2441,7 @@
         <v>14</v>
       </c>
       <c r="H33" s="17"/>
-      <c r="I33" s="17"/>
+      <c r="I33" s="45"/>
       <c r="J33" s="17"/>
       <c r="K33" s="17"/>
       <c r="L33" s="17"/>
@@ -2395,7 +2451,7 @@
       <c r="P33" s="36"/>
       <c r="Q33" s="32"/>
     </row>
-    <row r="34" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B34" s="39"/>
       <c r="C34" s="17"/>
       <c r="D34" s="17"/>
@@ -2408,7 +2464,7 @@
         <v>14</v>
       </c>
       <c r="H34" s="17"/>
-      <c r="I34" s="17"/>
+      <c r="I34" s="45"/>
       <c r="J34" s="17"/>
       <c r="K34" s="17"/>
       <c r="L34" s="17"/>
@@ -2418,7 +2474,7 @@
       <c r="P34" s="36"/>
       <c r="Q34" s="32"/>
     </row>
-    <row r="35" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B35" s="39"/>
       <c r="C35" s="17"/>
       <c r="D35" s="17"/>
@@ -2431,7 +2487,7 @@
         <v>14</v>
       </c>
       <c r="H35" s="17"/>
-      <c r="I35" s="17"/>
+      <c r="I35" s="45"/>
       <c r="J35" s="17"/>
       <c r="K35" s="17"/>
       <c r="L35" s="17"/>
@@ -2441,7 +2497,7 @@
       <c r="P35" s="36"/>
       <c r="Q35" s="32"/>
     </row>
-    <row r="36" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:17" x14ac:dyDescent="0.2">
       <c r="B36" s="39"/>
       <c r="C36" s="17"/>
       <c r="D36" s="17"/>
@@ -2454,7 +2510,7 @@
         <v>14</v>
       </c>
       <c r="H36" s="17"/>
-      <c r="I36" s="17"/>
+      <c r="I36" s="45"/>
       <c r="J36" s="17"/>
       <c r="K36" s="17"/>
       <c r="L36" s="17"/>
@@ -2464,7 +2520,7 @@
       <c r="P36" s="36"/>
       <c r="Q36" s="32"/>
     </row>
-    <row r="37" spans="2:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B37" s="41"/>
       <c r="C37" s="25"/>
       <c r="D37" s="25"/>

</xml_diff>

<commit_message>
CAD created, all drivertrain hardware ordered
</commit_message>
<xml_diff>
--- a/docs/financials/Buddy_BOM.xlsx
+++ b/docs/financials/Buddy_BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ventimaj/Desktop/Desktop - MacBook Air (263)/Buddy_Robot/docs/financials/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\venti\Desktop\Buddy_Robot\docs\financials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DA2F662-2898-A243-8BCD-A3C5B8DC8AB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C13E3E20-B09E-4437-8315-303E254DD92E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17420" xr2:uid="{C64966AC-B3BB-9844-956C-858996BC28CC}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{C64966AC-B3BB-9844-956C-858996BC28CC}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="128">
   <si>
     <t>Descriptive Part Name</t>
   </si>
@@ -329,6 +329,108 @@
   </si>
   <si>
     <t>Tri-band</t>
+  </si>
+  <si>
+    <t>Planetary Gear Motor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Encoder Cables: 4-Pos JST XH [MH-FC] to 4 x 1-Pos TJC8 [MH-FC] </t>
+  </si>
+  <si>
+    <t>goBILDA</t>
+  </si>
+  <si>
+    <t>Order Num: 200129494</t>
+  </si>
+  <si>
+    <t>5203 Series Yellow Jacket Planetary Gear
+Motor (26.9:1 Ratio, 24mm Length 8mm
+REX® Shaft, 223 RPM, 3.3 - 5V Encoder)</t>
+  </si>
+  <si>
+    <t>SKU: 3801-0919-0300</t>
+  </si>
+  <si>
+    <t>SKU: 5203-2402-0027</t>
+  </si>
+  <si>
+    <t>Encoder Breakout Cable (4-Pos JST XH
+[MH-FC] to 4 x 1-Pos TJC8 [MH-FC],
+300mm Length)</t>
+  </si>
+  <si>
+    <t>Motor to Driver Power Cables</t>
+  </si>
+  <si>
+    <t>SKU: 3800-0013-0300</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.5mm Bullet Lead (MH-FC, 300mm Length) </t>
+  </si>
+  <si>
+    <t>Wheel Hub (Sonic)</t>
+  </si>
+  <si>
+    <t>SKU: 1309-0016-4008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1309 Series Sonic Hub (8mm REX® Bore) </t>
+  </si>
+  <si>
+    <t>M4 Socket 12mm (24 pack)</t>
+  </si>
+  <si>
+    <t>SKU: 2822-0004-0012</t>
+  </si>
+  <si>
+    <t>Premium M4 Socket Head Thread-Locking
+Screw (12mm Length) - 25 Pack</t>
+  </si>
+  <si>
+    <t>Traction Wheel</t>
+  </si>
+  <si>
+    <t>SKU: 3626-0014-0096</t>
+  </si>
+  <si>
+    <t>Hogback Traction Wheel (96mm Diameter,
+50A Durometer)</t>
+  </si>
+  <si>
+    <t>https://www.gobilda.com/5203-series-yellow-jacket-planetary-gear-motor-26-9-1-ratio-24mm-length-8mm-rex-shaft-223-rpm-3-3-5v-encoder/</t>
+  </si>
+  <si>
+    <t>https://www.gobilda.com/encoder-breakout-cable-4-pos-jst-xh-mh-fc-to-4-x-1-pos-tjc8-mh-fc-300mm-length/</t>
+  </si>
+  <si>
+    <t>https://www.gobilda.com/3-5mm-bullet-lead-mh-fc-300mm-length/</t>
+  </si>
+  <si>
+    <t>https://www.gobilda.com/1309-series-sonic-hub-8mm-rex-bore/</t>
+  </si>
+  <si>
+    <t>https://www.gobilda.com/hogback-traction-wheel-96mm-diameter-50a-durometer/</t>
+  </si>
+  <si>
+    <t>https://www.gobilda.com/premium-m4-socket-head-thread-locking-screw-12mm-length-25-pack/</t>
+  </si>
+  <si>
+    <t>Motor Driver Carrier</t>
+  </si>
+  <si>
+    <t>Pololu</t>
+  </si>
+  <si>
+    <t>Item Number: 1451</t>
+  </si>
+  <si>
+    <t>https://www.pololu.com/product/1451</t>
+  </si>
+  <si>
+    <t>Salesorder 1J592793</t>
+  </si>
+  <si>
+    <t>VNH5019 Motor Driver Carrier: operates from 5.5 to 24 V and can deliver a continuous 12 A (30 A peak). It works with 2.5 to 5 V logic levels, supports ultrasonic (up to 20 kHz) PWM, and features current sense feedback (an analog voltage proportional to the motor current). Along with built-in protection against reverse-voltage, over-voltage, under-voltage, over-temperature, and over-current</t>
   </si>
 </sst>
 </file>
@@ -668,7 +770,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -824,6 +926,18 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1310,21 +1424,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3B39B8B-F33B-1140-8548-5838830ED406}">
   <dimension ref="B1:V37"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="31" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.125" bestFit="1" customWidth="1"/>
     <col min="7" max="9" width="16.5" customWidth="1"/>
     <col min="10" max="11" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="15" max="16" width="24.83203125" customWidth="1"/>
+    <col min="15" max="16" width="24.875" customWidth="1"/>
     <col min="17" max="17" width="46.5" customWidth="1"/>
-    <col min="19" max="19" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="25.6640625" customWidth="1"/>
-    <col min="22" max="22" width="33.1640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="25.625" customWidth="1"/>
+    <col min="22" max="22" width="33.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:22" ht="29" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:22" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1379,7 +1493,7 @@
       <c r="T2" s="48"/>
       <c r="U2" s="7"/>
     </row>
-    <row r="3" spans="2:22" ht="61" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:22" ht="60.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="B3" s="39" t="s">
         <v>31</v>
       </c>
@@ -1435,7 +1549,7 @@
       </c>
       <c r="U3" s="7"/>
     </row>
-    <row r="4" spans="2:22" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:22" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="39" t="s">
         <v>37</v>
       </c>
@@ -1483,7 +1597,7 @@
       <c r="T4" s="7"/>
       <c r="U4" s="7"/>
     </row>
-    <row r="5" spans="2:22" ht="75" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:22" ht="75" x14ac:dyDescent="0.25">
       <c r="B5" s="40" t="s">
         <v>57</v>
       </c>
@@ -1529,7 +1643,7 @@
       <c r="T5" s="49"/>
       <c r="U5" s="7"/>
     </row>
-    <row r="6" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B6" s="39" t="s">
         <v>59</v>
       </c>
@@ -1563,7 +1677,7 @@
       <c r="T6" s="46"/>
       <c r="U6" s="7"/>
     </row>
-    <row r="7" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B7" s="39" t="s">
         <v>60</v>
       </c>
@@ -1597,7 +1711,7 @@
       <c r="T7" s="50"/>
       <c r="U7" s="7"/>
     </row>
-    <row r="8" spans="2:22" ht="60" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:22" ht="60" x14ac:dyDescent="0.25">
       <c r="B8" s="5" t="s">
         <v>61</v>
       </c>
@@ -1651,7 +1765,7 @@
       <c r="T8" s="51"/>
       <c r="U8" s="7"/>
     </row>
-    <row r="9" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B9" s="5" t="s">
         <v>67</v>
       </c>
@@ -1705,7 +1819,7 @@
       <c r="T9" s="52"/>
       <c r="U9" s="7"/>
     </row>
-    <row r="10" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B10" s="5" t="s">
         <v>71</v>
       </c>
@@ -1759,7 +1873,7 @@
       <c r="T10" s="53"/>
       <c r="U10" s="7"/>
     </row>
-    <row r="11" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B11" s="5" t="s">
         <v>77</v>
       </c>
@@ -1812,7 +1926,7 @@
       <c r="T11" s="54"/>
       <c r="U11" s="7"/>
     </row>
-    <row r="12" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B12" s="5" t="s">
         <v>82</v>
       </c>
@@ -1866,7 +1980,7 @@
       <c r="T12" s="55"/>
       <c r="U12" s="7"/>
     </row>
-    <row r="13" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B13" s="5" t="s">
         <v>87</v>
       </c>
@@ -1909,7 +2023,7 @@
       <c r="T13" s="56"/>
       <c r="U13" s="7"/>
     </row>
-    <row r="14" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:22" ht="30" x14ac:dyDescent="0.25">
       <c r="B14" s="5" t="s">
         <v>90</v>
       </c>
@@ -1938,7 +2052,7 @@
       <c r="J14" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="K14" s="17" t="s">
+      <c r="K14" s="5" t="s">
         <v>94</v>
       </c>
       <c r="L14" s="17"/>
@@ -1949,11 +2063,14 @@
       <c r="O14" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="P14" s="36" t="s">
+      <c r="P14" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="Q14" s="32" t="s">
+      <c r="Q14" s="61" t="s">
         <v>92</v>
+      </c>
+      <c r="R14" t="s">
+        <v>15</v>
       </c>
       <c r="S14" s="57" t="s">
         <v>16</v>
@@ -1961,192 +2078,333 @@
       <c r="T14" s="57"/>
       <c r="U14" s="7"/>
     </row>
-    <row r="15" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B15" s="5"/>
-      <c r="C15" s="17"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="19" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+    <row r="15" spans="2:22" ht="45" x14ac:dyDescent="0.25">
+      <c r="B15" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C15" s="17">
+        <v>4</v>
+      </c>
+      <c r="D15" s="17">
+        <v>4</v>
+      </c>
+      <c r="E15" s="18">
+        <f>(219.96 + (219.96/322.09)*(11.99+24.97))/4</f>
+        <v>61.300131950697015</v>
+      </c>
+      <c r="F15" s="19">
+        <f t="shared" si="0"/>
+        <v>245.20052780278806</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="H15" s="42"/>
+        <v>26</v>
+      </c>
+      <c r="H15" s="42">
+        <v>46232</v>
+      </c>
       <c r="I15" s="45"/>
-      <c r="J15" s="17"/>
-      <c r="K15" s="17"/>
+      <c r="J15" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>102</v>
+      </c>
       <c r="L15" s="17"/>
       <c r="M15" s="17"/>
       <c r="N15" s="5"/>
-      <c r="O15" s="24"/>
-      <c r="P15" s="22"/>
-      <c r="Q15" s="32"/>
+      <c r="O15" s="24" t="s">
+        <v>116</v>
+      </c>
+      <c r="P15" s="59" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q15" s="61" t="s">
+        <v>100</v>
+      </c>
+      <c r="R15" t="s">
+        <v>15</v>
+      </c>
       <c r="S15" s="47" t="s">
         <v>14</v>
       </c>
       <c r="T15" s="47"/>
       <c r="U15" s="7"/>
     </row>
-    <row r="16" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B16" s="5"/>
-      <c r="C16" s="17"/>
-      <c r="D16" s="17"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="19" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+    <row r="16" spans="2:22" ht="45" x14ac:dyDescent="0.25">
+      <c r="B16" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="C16" s="17">
+        <v>4</v>
+      </c>
+      <c r="D16" s="17">
+        <v>4</v>
+      </c>
+      <c r="E16" s="18">
+        <f>(15.96 + (15.96/322.09)*(11.99+24.97))/4</f>
+        <v>4.4478546369027292</v>
+      </c>
+      <c r="F16" s="19">
+        <f t="shared" si="0"/>
+        <v>17.791418547610917</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="H16" s="42"/>
+        <v>26</v>
+      </c>
+      <c r="H16" s="42">
+        <v>46232</v>
+      </c>
       <c r="I16" s="45"/>
-      <c r="J16" s="29"/>
-      <c r="K16" s="17"/>
+      <c r="J16" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>101</v>
+      </c>
       <c r="L16" s="17"/>
       <c r="M16" s="17"/>
       <c r="N16" s="5"/>
-      <c r="O16" s="20"/>
-      <c r="P16" s="35"/>
-      <c r="Q16" s="32"/>
+      <c r="O16" s="24" t="s">
+        <v>117</v>
+      </c>
+      <c r="P16" s="59" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q16" s="61" t="s">
+        <v>103</v>
+      </c>
       <c r="U16" s="7"/>
       <c r="V16" s="7"/>
     </row>
-    <row r="17" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B17" s="5"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="17"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="19" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+    <row r="17" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B17" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="C17" s="16">
+        <v>4</v>
+      </c>
+      <c r="D17" s="17">
+        <v>4</v>
+      </c>
+      <c r="E17" s="18">
+        <f>(9.96 + (9.96/322.09)*(11.99+24.97))/4</f>
+        <v>2.7757288335558385</v>
+      </c>
+      <c r="F17" s="19">
+        <f t="shared" si="0"/>
+        <v>11.102915334223354</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="H17" s="42"/>
+        <v>26</v>
+      </c>
+      <c r="H17" s="42">
+        <v>46232</v>
+      </c>
       <c r="I17" s="45"/>
-      <c r="J17" s="17"/>
-      <c r="K17" s="17"/>
+      <c r="J17" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>105</v>
+      </c>
       <c r="L17" s="17"/>
       <c r="M17" s="17"/>
       <c r="N17" s="5"/>
-      <c r="O17" s="24"/>
-      <c r="P17" s="22"/>
-      <c r="Q17" s="32"/>
+      <c r="O17" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="P17" s="59" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q17" s="32" t="s">
+        <v>106</v>
+      </c>
       <c r="S17" s="7"/>
       <c r="V17" s="7"/>
     </row>
-    <row r="18" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B18" s="5"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="17"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="19" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+    <row r="18" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B18" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C18" s="17">
+        <v>4</v>
+      </c>
+      <c r="D18" s="17">
+        <v>4</v>
+      </c>
+      <c r="E18" s="18">
+        <f>(31.96 + (31.96/322.09)*(11.99+24.97))/4</f>
+        <v>8.9068567791611049</v>
+      </c>
+      <c r="F18" s="19">
+        <f t="shared" si="0"/>
+        <v>35.627427116644419</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="H18" s="42"/>
+        <v>26</v>
+      </c>
+      <c r="H18" s="42">
+        <v>46232</v>
+      </c>
       <c r="I18" s="45"/>
-      <c r="J18" s="17"/>
-      <c r="K18" s="17"/>
+      <c r="J18" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="K18" s="5" t="s">
+        <v>108</v>
+      </c>
       <c r="L18" s="17"/>
       <c r="M18" s="17"/>
       <c r="N18" s="5"/>
-      <c r="O18" s="23"/>
-      <c r="P18" s="36"/>
-      <c r="Q18" s="32"/>
+      <c r="O18" s="24" t="s">
+        <v>119</v>
+      </c>
+      <c r="P18" s="59" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q18" s="32" t="s">
+        <v>109</v>
+      </c>
       <c r="S18" s="7"/>
       <c r="V18" s="7"/>
     </row>
-    <row r="19" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B19" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="C19" s="16"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="19" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+    <row r="19" spans="2:22" ht="30" x14ac:dyDescent="0.25">
+      <c r="B19" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="C19" s="16">
+        <v>1</v>
+      </c>
+      <c r="D19" s="17">
+        <v>1</v>
+      </c>
+      <c r="E19" s="18">
+        <f>4.29 + (4.29/322.09)*(11.99+24.97)</f>
+        <v>4.782279797572107</v>
+      </c>
+      <c r="F19" s="19">
+        <f t="shared" si="0"/>
+        <v>4.782279797572107</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="H19" s="42"/>
+        <v>26</v>
+      </c>
+      <c r="H19" s="42">
+        <v>46232</v>
+      </c>
       <c r="I19" s="45"/>
-      <c r="J19" s="17"/>
-      <c r="K19" s="17"/>
+      <c r="J19" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>111</v>
+      </c>
       <c r="L19" s="17"/>
       <c r="M19" s="17"/>
       <c r="N19" s="5"/>
-      <c r="O19" s="23"/>
-      <c r="P19" s="36"/>
-      <c r="Q19" s="32"/>
+      <c r="O19" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="P19" s="59" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q19" s="31" t="s">
+        <v>112</v>
+      </c>
       <c r="S19" s="7"/>
       <c r="V19" s="7"/>
     </row>
-    <row r="20" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B20" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="C20" s="16"/>
-      <c r="D20" s="17"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="19" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+    <row r="20" spans="2:22" ht="30" x14ac:dyDescent="0.25">
+      <c r="B20" s="60" t="s">
+        <v>113</v>
+      </c>
+      <c r="C20" s="16">
+        <v>4</v>
+      </c>
+      <c r="D20" s="17">
+        <v>4</v>
+      </c>
+      <c r="E20" s="18">
+        <f>(39.96 + (39.96/322.09)*(11.99+24.97))/4</f>
+        <v>11.136357850290292</v>
+      </c>
+      <c r="F20" s="19">
+        <f t="shared" si="0"/>
+        <v>44.545431401161167</v>
       </c>
       <c r="G20" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="H20" s="42"/>
+        <v>26</v>
+      </c>
+      <c r="H20" s="42">
+        <v>46232</v>
+      </c>
       <c r="I20" s="45"/>
-      <c r="J20" s="29"/>
-      <c r="K20" s="17"/>
+      <c r="J20" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="K20" s="5" t="s">
+        <v>114</v>
+      </c>
       <c r="L20" s="17"/>
       <c r="M20" s="17"/>
       <c r="N20" s="5"/>
-      <c r="O20" s="20"/>
-      <c r="P20" s="35"/>
-      <c r="Q20" s="32"/>
+      <c r="O20" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="P20" s="59" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q20" s="31" t="s">
+        <v>115</v>
+      </c>
       <c r="S20" s="7"/>
       <c r="V20" s="7"/>
     </row>
-    <row r="21" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B21" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="C21" s="17"/>
-      <c r="D21" s="17"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="19" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+    <row r="21" spans="2:22" ht="105" x14ac:dyDescent="0.25">
+      <c r="B21" s="60" t="s">
+        <v>122</v>
+      </c>
+      <c r="C21" s="17">
+        <v>4</v>
+      </c>
+      <c r="D21" s="17">
+        <v>4</v>
+      </c>
+      <c r="E21" s="18">
+        <f>85.98/4</f>
+        <v>21.495000000000001</v>
+      </c>
+      <c r="F21" s="19">
+        <f t="shared" si="0"/>
+        <v>85.98</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="H21" s="29"/>
+        <v>26</v>
+      </c>
+      <c r="H21" s="42">
+        <v>46232</v>
+      </c>
       <c r="I21" s="45"/>
-      <c r="J21" s="29"/>
-      <c r="K21" s="17"/>
+      <c r="J21" s="29" t="s">
+        <v>123</v>
+      </c>
+      <c r="K21" s="5" t="s">
+        <v>124</v>
+      </c>
       <c r="L21" s="17"/>
       <c r="M21" s="17"/>
       <c r="N21" s="5"/>
-      <c r="O21" s="20"/>
-      <c r="P21" s="35"/>
-      <c r="Q21" s="32"/>
-    </row>
-    <row r="22" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B22" s="39" t="s">
-        <v>45</v>
-      </c>
+      <c r="O21" s="24" t="s">
+        <v>125</v>
+      </c>
+      <c r="P21" s="59" t="s">
+        <v>126</v>
+      </c>
+      <c r="Q21" s="31" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="22" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C22" s="16"/>
       <c r="D22" s="17"/>
       <c r="E22" s="18"/>
@@ -2168,10 +2426,7 @@
       <c r="P22" s="36"/>
       <c r="Q22" s="32"/>
     </row>
-    <row r="23" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="39" t="s">
-        <v>46</v>
-      </c>
+    <row r="23" spans="2:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C23" s="17"/>
       <c r="D23" s="17"/>
       <c r="E23" s="18"/>
@@ -2193,10 +2448,7 @@
       <c r="P23" s="35"/>
       <c r="Q23" s="32"/>
     </row>
-    <row r="24" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B24" s="39" t="s">
-        <v>47</v>
-      </c>
+    <row r="24" spans="2:22" x14ac:dyDescent="0.25">
       <c r="C24" s="16"/>
       <c r="D24" s="17"/>
       <c r="E24" s="18"/>
@@ -2224,10 +2476,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="25" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="39" t="s">
-        <v>48</v>
-      </c>
+    <row r="25" spans="2:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C25" s="17"/>
       <c r="D25" s="17"/>
       <c r="E25" s="18"/>
@@ -2253,11 +2502,13 @@
       </c>
       <c r="T25" s="13">
         <f>SUM(F3:F37)</f>
-        <v>728.82000000000016</v>
-      </c>
-    </row>
-    <row r="26" spans="2:22" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="39"/>
+        <v>1173.8500000000001</v>
+      </c>
+    </row>
+    <row r="26" spans="2:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="C26" s="16"/>
       <c r="D26" s="17"/>
       <c r="E26" s="18"/>
@@ -2283,11 +2534,13 @@
       </c>
       <c r="T26" s="15">
         <f>T24-T25</f>
-        <v>1271.1799999999998</v>
-      </c>
-    </row>
-    <row r="27" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B27" s="39"/>
+        <v>826.14999999999986</v>
+      </c>
+    </row>
+    <row r="27" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B27" s="5" t="s">
+        <v>43</v>
+      </c>
       <c r="C27" s="17"/>
       <c r="D27" s="17"/>
       <c r="E27" s="18"/>
@@ -2309,9 +2562,9 @@
       <c r="P27" s="35"/>
       <c r="Q27" s="32"/>
     </row>
-    <row r="28" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B28" s="39" t="s">
-        <v>49</v>
+    <row r="28" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B28" s="5" t="s">
+        <v>44</v>
       </c>
       <c r="C28" s="16"/>
       <c r="D28" s="17"/>
@@ -2334,9 +2587,9 @@
       <c r="P28" s="36"/>
       <c r="Q28" s="32"/>
     </row>
-    <row r="29" spans="2:22" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B29" s="39" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C29" s="17"/>
       <c r="D29" s="17"/>
@@ -2359,8 +2612,10 @@
       <c r="P29" s="36"/>
       <c r="Q29" s="32"/>
     </row>
-    <row r="30" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B30" s="39"/>
+    <row r="30" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B30" s="39" t="s">
+        <v>46</v>
+      </c>
       <c r="C30" s="16"/>
       <c r="D30" s="17"/>
       <c r="E30" s="18"/>
@@ -2382,8 +2637,10 @@
       <c r="P30" s="36"/>
       <c r="Q30" s="32"/>
     </row>
-    <row r="31" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B31" s="39"/>
+    <row r="31" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B31" s="39" t="s">
+        <v>47</v>
+      </c>
       <c r="C31" s="17"/>
       <c r="D31" s="17"/>
       <c r="E31" s="18"/>
@@ -2405,8 +2662,10 @@
       <c r="P31" s="36"/>
       <c r="Q31" s="32"/>
     </row>
-    <row r="32" spans="2:22" x14ac:dyDescent="0.2">
-      <c r="B32" s="39"/>
+    <row r="32" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B32" s="39" t="s">
+        <v>48</v>
+      </c>
       <c r="C32" s="17"/>
       <c r="D32" s="17"/>
       <c r="E32" s="18"/>
@@ -2428,7 +2687,7 @@
       <c r="P32" s="36"/>
       <c r="Q32" s="32"/>
     </row>
-    <row r="33" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B33" s="39"/>
       <c r="C33" s="16"/>
       <c r="D33" s="17"/>
@@ -2451,7 +2710,7 @@
       <c r="P33" s="36"/>
       <c r="Q33" s="32"/>
     </row>
-    <row r="34" spans="2:17" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B34" s="39"/>
       <c r="C34" s="17"/>
       <c r="D34" s="17"/>
@@ -2474,8 +2733,10 @@
       <c r="P34" s="36"/>
       <c r="Q34" s="32"/>
     </row>
-    <row r="35" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B35" s="39"/>
+    <row r="35" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B35" s="39" t="s">
+        <v>49</v>
+      </c>
       <c r="C35" s="17"/>
       <c r="D35" s="17"/>
       <c r="E35" s="18"/>
@@ -2497,8 +2758,10 @@
       <c r="P35" s="36"/>
       <c r="Q35" s="32"/>
     </row>
-    <row r="36" spans="2:17" x14ac:dyDescent="0.2">
-      <c r="B36" s="39"/>
+    <row r="36" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="B36" s="39" t="s">
+        <v>50</v>
+      </c>
       <c r="C36" s="17"/>
       <c r="D36" s="17"/>
       <c r="E36" s="18"/>
@@ -2520,7 +2783,7 @@
       <c r="P36" s="36"/>
       <c r="Q36" s="32"/>
     </row>
-    <row r="37" spans="2:17" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:17" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B37" s="41"/>
       <c r="C37" s="25"/>
       <c r="D37" s="25"/>
@@ -2619,7 +2882,7 @@
       <formula>G4=$AC$2</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3:G37" xr:uid="{E79D009E-1FC5-344B-B22B-A284ED74F5B4}">
       <formula1>$S$6:$S$15</formula1>
     </dataValidation>
@@ -2632,6 +2895,13 @@
     <hyperlink ref="O5" r:id="rId5" display="https://vilros.com/products/vilros-soldering-iron-kit-electronics-14-in-1-60w-adjustable-temperature-soldering-iron-with-on-off-switch-5pcs-soldering-iron-tips-desoldering-pump-tweezers-stand-solder-pu-carry-bag?variant=31184817684574&amp;country=US&amp;currency=USD&amp;utm_medium=product_sync&amp;utm_source=google&amp;utm_content=sag_organic&amp;utm_campaign=sag_organic&amp;tw_source=google&amp;tw_adid=&amp;tw_campaign=18070425970&amp;gad_source=1&amp;gad_campaignid=17177576781&amp;gbraid=0AAAAAD1QJAhpwOz4TG9imhRizOjsiF33r&amp;gclid=Cj0KCQjwr4jSBhCSARIsAOX1E-IcDf7VArvc12fU96XQu_eogR6Cku3p0W322S9UE6enAxh-gCdhcRkaApEYEALw_wcB" xr:uid="{F8EE24A7-3DF2-4835-8818-4CF5FD2EFD11}"/>
     <hyperlink ref="O8" r:id="rId6" xr:uid="{ED02DEDC-B0EC-0749-B7B9-A7D73B4129EF}"/>
     <hyperlink ref="O9" r:id="rId7" xr:uid="{5B52362B-868D-40C8-ADAC-0C067B706503}"/>
+    <hyperlink ref="O15" r:id="rId8" xr:uid="{8A4421D2-6527-42C4-9794-8C1C34D959C5}"/>
+    <hyperlink ref="O16" r:id="rId9" xr:uid="{71C4DB52-47C3-49A4-A2B6-88F733F311B8}"/>
+    <hyperlink ref="O17" r:id="rId10" xr:uid="{FE6BD667-D201-4908-878D-D55FF2DE92E9}"/>
+    <hyperlink ref="O18" r:id="rId11" xr:uid="{C3E0327B-C273-4E62-98EA-3FF38BD4F4B9}"/>
+    <hyperlink ref="O20" r:id="rId12" xr:uid="{91A94F13-5311-47E0-9354-A5682DCC5DAC}"/>
+    <hyperlink ref="O19" r:id="rId13" xr:uid="{FF128169-492B-4115-BDF8-082DC0D10945}"/>
+    <hyperlink ref="O21" r:id="rId14" xr:uid="{CF446E74-EC60-4FB5-9653-043616385554}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>